<commit_message>
Cleanup large file from history and update data
</commit_message>
<xml_diff>
--- a/NEWS/market_news.xlsx
+++ b/NEWS/market_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,22 +463,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Doanh nghiệp Mỹ hưởng lợi gì khi cùng ông Trump tới Trung Quốc?</t>
+          <t>Chứng khoán Mỹ lập kỷ lục nhờ cổ phiếu công nghệ, giá dầu giảm vì mối lo lãi suất cao hơn lâu hơn</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Trong khi Boeing và Cargill có thể đạt thỏa thuận mua hàng, Nvidia, Meta và Tesla lại đến Trung Quốc để giải quyết các rào cản chính sách tại đây.</t>
+          <t>Thị trường chứng kho#225;n Mỹ tăng điểm trong phi#234;n giao dịch ng#224;y thứ Tư (13/5), khi cổ phiếu c#244;ng nghệ được mua mạnh, đưa hai chỉ số Samp;P 500 v#224; Nasdaq lập kỷ lục mới...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 11:18:27 +0700</t>
+          <t>Thu, 14 May 2026 01:18:51 GMT</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -486,29 +486,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/doanh-nghiep-my-huong-loi-gi-khi-cung-ong-trump-toi-trung-quoc-5073296.html</t>
+          <t>https://vneconomy.vn/chung-khoan-my-lap-ky-luc-nho-co-phieu-cong-nghe-gia-dau-giam-vi-moi-lo-lai-suat-cao-hon-lau-hon.htm</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lãi suất tiết kiệm ngân hàng nào cao nhất?</t>
+          <t>Áp lực lạm phát đè nặng giá vàng, SPDR Gold Trust mua ròng liên tục</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lãi suất tiết kiệm hạ nhiệt sau chỉ đạo của Thống đốc song mặt bằng chung với các khoản thỏa thuận vẫn ở mức hấp dẫn, một số nhà băng trả 8-9% một năm.</t>
+          <t>Gi#225; v#224;ng thế giới giảm trong phi#234;n giao dịch ng#224;y thứ Tư (13/5), trượt khỏi mốc 4.700 USD/oz, khi #225;p lực lạm ph#225;t gia tăng ở Mỹ đẩy cao mối lo l#227;i suất cao hơn l#226;u hơn...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 05:33:34 +0700</t>
+          <t>Thu, 14 May 2026 00:26:34 GMT</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -516,29 +516,29 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/lai-suat-tiet-kiem-ngan-hang-nao-cao-nhat-5072646.html</t>
+          <t>https://vneconomy.vn/ap-luc-lam-phat-de-nang-gia-vang-spdr-gold-trust-mua-rong-lien-tuc.htm</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Giá vàng tuần này có thể tăng</t>
+          <t>Theo dấu dòng tiền cá mập 13/05: Khối ngoại bán ròng phiên thứ mười bốn liên tiếp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tiếp đà phục hồi tuần qua, Phố Wall lẫn nhà đầu tư cá nhân cùng dự báo giá vàng tăng, với kỳ vọng hạ nhiệt căng thẳng Mỹ - Iran.</t>
+          <t>Trong phiên rung lắc của thị trường, cả khối tự doanh và khối ngoại đều bán ròng.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 00:00:00 +0700</t>
+          <t>Wed, 13 May 2026 19:00:32 +0700</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/gia-vang-tuan-nay-co-the-tang-5072198.html</t>
+          <t>http://vietstock.vn/2026/05/theo-dau-dong-tien-ca-map-1305-khoi-ngoai-ban-rong-phien-thu-muoi-bon-lien-tiep-830-1442280.htm</t>
         </is>
       </c>
     </row>
@@ -558,17 +558,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MSCI và FTSE khác nhau thế nào trong nâng hạng thị trường chứng khoán?</t>
+          <t>Phó thủ tướng: FDI thế hệ mới phải tạo giá trị cho Việt Nam</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cùng là nâng hạng thị trường chứng khoán, nhưng MSCI và FTSE có tiêu chí, tầm ảnh hưởng và sức hấp dẫn khác nhau.</t>
+          <t>Việt Nam không thu hút vốn FDI bằng mọi giá, mà ưu tiên các dự án công nghệ có khả năng kết nối doanh nghiệp nội.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sun, 10 May 2026 00:02:00 +0700</t>
+          <t>Wed, 13 May 2026 19:00:10 +0700</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -576,29 +576,29 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/msci-va-ftse-khac-nhau-the-nao-trong-nang-hang-thi-truong-chung-khoan-5070886.html</t>
+          <t>https://vnexpress.net/pho-thu-tuong-fdi-the-he-moi-phai-tao-gia-tri-cho-viet-nam-5073553.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CEO Nvidia, Apple sẽ cùng ông Trump đến Trung Quốc</t>
+          <t>FDI thế hệ mới cần cùng Việt Nam tạo ra giá trị mới, năng lực mới, vị thế mới</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hơn 10 lãnh đạo doanh nghiệp, trong đó có CEO Nvidia, Apple, Qualcomm, Citigroup và Boeing sẽ cùng Tổng thống Mỹ đến Trung Quốc tuần tới.</t>
+          <t>Phát biểu tại Diễn đàn Nhịp cầu Phát triển Việt Nam 2026 chiều nay, 13/5, Phó Thủ tướng Nguyễn Văn Thắng nhấn mạnh, FDI thế hệ mới không chỉ đến Việt Nam để sản xuất, để khai thác thị trường, mà cần cùng Việt Nam tạo ra giá trị mới, năng lực mới và vị thế mới trong chuỗi giá trị toàn cầu.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sat, 09 May 2026 00:00:00 +0700</t>
+          <t>Wed, 13 May 26 17:30:00 +0700</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/ceo-nvidia-apple-se-cung-ong-trump-den-trung-quoc-5071620.html</t>
+          <t>https://cafef.vn/fdi-the-he-moi-can-cung-viet-nam-tao-ra-gia-tri-moi-nang-luc-moi-vi-the-moi-188260513165309213.chn</t>
         </is>
       </c>
     </row>
@@ -618,17 +618,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Thủ tướng Sri Lanka muốn doanh nghiệp Việt tăng hợp tác thương mại, hàng không</t>
+          <t>Doanh nghiệp Mỹ hưởng lợi gì khi cùng ông Trump tới Trung Quốc?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thủ tướng Sri Lanka muốn doanh nghiệp Việt mở rộng hợp tác trong lĩnh vực thương mại, chế biến thực phẩm, logistics, hàng không và du lịch.</t>
+          <t>Trong khi Boeing và Cargill có thể đạt thỏa thuận mua hàng, Nvidia, Meta và Tesla lại đến Trung Quốc để giải quyết các rào cản chính sách tại đây.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 21:48:02 +0700</t>
+          <t>Wed, 13 May 2026 11:18:27 +0700</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -636,569 +636,569 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/thu-tuong-sri-lanka-muon-doanh-nghiep-viet-tang-hop-tac-thuong-mai-hang-khong-5071709.html</t>
+          <t>https://vnexpress.net/doanh-nghiep-my-huong-loi-gi-khi-cung-ong-trump-toi-trung-quoc-5073296.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Công bố giá xăng E10 Petrolimex</t>
+          <t>Tỷ giá đồng yên biến động mạnh trong lúc Bộ trưởng Bessent thăm Nhật Bản</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tập đoàn Xăng dầu Việt Nam (Petrolimex) vừa thông báo giá bán xăng sinh học E10 RON 95 áp dụng từ ngày 0h ngày 13/5. Theo đó, giá bán xăng sinh học E10 RON 95-V tại cửa hàng xăng dầu tại thị trường vùng 1 là 24.630 đồng/lít, tại các thị trường vùng 2 là 25.120 đồng/lít.</t>
+          <t>Giới chức Nhật Bản vốn tin rằng một sự ủng hộ từ #244;ng Bessent sẽ gi#250;p củng cố t#225;c dụng của việc họ can thiệp v#224;o thị trường tiền tệ, theo đ#243; cản lại #225;p lực mất gi#225; đồng y#234;n...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 16:45:00 +0700</t>
+          <t>Wed, 13 May 2026 03:47:17 GMT</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://cafef.vn/cong-bo-gia-xang-e10-petrolimex-188260513154754794.chn</t>
+          <t>https://vneconomy.vn/ty-gia-dong-yen-bien-dong-manh-trong-luc-bo-truong-bessent-tham-nhat-ban.htm</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cổ phiếu dầu khí hút tiền nhà đầu tư trong nước</t>
+          <t>Lạm phát ở Mỹ cao nhất gần 3 năm do giá xăng dầu tăng mạnh, Fed gặp khó</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Toàn bộ cổ phiếu dầu khí bật mạnh, trong đó GAS chạm trần và dẫn đầu danh sách "trụ đỡ" của VN-Index trước áp lực xả hàng cổ phiếu Vingroup.</t>
+          <t>Giới chuy#234;n gia cảnh b#225;o rằng gi#225; cả ở nền kinh tế lớn nhất thế giới sẽ tiếp tục leo thang tr#234;n phạm vi ng#224;y c#224;ng rộng hơn trong những th#225;ng sắp tới, khiến Fed kh#243; hạ l#227;i suất...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 16:25:11 +0700</t>
+          <t>Wed, 13 May 2026 02:04:51 GMT</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/co-phieu-dau-khi-hut-tien-nha-dau-tu-trong-nuoc-5073515.html</t>
+          <t>https://vneconomy.vn/lam-phat-o-my-cao-nhat-gan-3-nam-do-gia-xang-dau-tang-manh-fed-gap-kho.htm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chứng khoán 13-5: Điều gì khiến cổ phiếu dầu khí bùng nổ?</t>
+          <t>Dự báo MSCI đưa thị trường Việt Nam vào danh sách theo dõi trong năm 2026-2027</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Phiên giao dịch ngày 13-5 ghi nhận diễn biến đầy biến động của thị trường chứng khoán khi áp lực bán mạnh xuất hiện ở nhóm cổ phiếu vốn hóa lớn</t>
+          <t>Trong kịch bản cơ sở, BSC Research dự b#225;o thị trường chứng kho#225;n Việt Nam c#243; thể được MSCI th#244;ng b#225;o đưa v#224;o danh s#225;ch theo d#245;i (Watch-list) trong giai đoạn 2026-2027.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 16:14:00 +0700</t>
+          <t>Wed, 13 May 2026 01:57:58 GMT</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://cafef.vn/chung-khoan-13-5-dieu-gi-khien-co-phieu-dau-khi-bung-no-18826051316143265.chn</t>
+          <t>https://vneconomy.vn/du-bao-msci-dua-thi-truong-viet-nam-vao-danh-sach-theo-doi-trong-nam-2026-2027.htm</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SSIAM bắt tay 2 định chế tài chính, mở rộng cơ hội đầu tư và tài trợ vốn giữa Nhật Bản và Việt Nam</t>
+          <t>Chứng khoán Mỹ trượt khỏi kỷ lục sau báo cáo lạm phát, giá dầu tiếp tục leo thang</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Phát huy chuyên môn, mạng lưới và nguồn lực của từng bên, SSIAM, CCIX và DCI sẽ chủ động tìm kiếm, cấu trúc và triển khai các cơ hội đầu tư và tài trợ vốn trung, dài hạn, góp phần thúc đẩy tăng trưởng bền vững cho doanh nghiệp Việt Nam và nền kinh tế.</t>
+          <t>Mối lo về lạm ph#225;t phủ b#243;ng l#234;n t#226;m tr#237; nh#224; đầu tư ở Phố Wall trong phi#234;n n#224;y...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 13:53:00 +0700</t>
+          <t>Wed, 13 May 2026 01:18:43 GMT</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://cafef.vn/ssiam-bat-tay-2-dinh-che-tai-chinh-mo-rong-co-hoi-dau-tu-va-tai-tro-von-giua-nhat-ban-va-viet-nam-188260513135311114.chn</t>
+          <t>https://vneconomy.vn/chung-khoan-my-truot-khoi-ky-luc-sau-bao-cao-lam-phat-gia-dau-tiep-tuc-leo-thang.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FPT báo lãi tháng 4/2026 tăng 21%</t>
+          <t>Khối ngoại bán ròng hơn 800 tỷ, chủ yếu xả cổ phiếu ngân hàng</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FPT cho biết khối lượng đơn hàng ký mới tại thị trường nước ngoài đã tăng vọt 30% so với cùng kỳ.</t>
+          <t>Khối ngoại tiếp tục b#225;n r#242;ng 836.0 tỷ đồng, t#237;nh ri#234;ng giao dịch khớp lệnh th#236; họ b#225;n r#242;ng 685.3 tỷ đồng.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 12:03:00 +0700</t>
+          <t>Tue, 12 May 2026 14:06:05 GMT</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://cafef.vn/fpt-bao-lai-thang-4-2026-tang-21-188260513120329893.chn</t>
+          <t>https://vneconomy.vn/khoi-ngoai-ban-rong-hon-800-ty-chu-yeu-xa-co-phieu-ngan-hang.htm</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chủ tịch Đoàn Nguyên Đức gom thêm cổ phiếu HAG</t>
+          <t>Chứng khoán Mỹ vẫn lập đỉnh mới dù đàm phán hòa bình bế tắc, giá dầu tăng 3%</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ông Đoàn Nguyên Đức- Chủ tịch HĐQT Hoàng Anh Gia Lai, đã mua vào 4 triệu cổ phiếu HAG bằng phương thức khớp lệnh trên sàn, qua đó nâng sở hữu lên 25,09%.</t>
+          <t>“Với sự b#249;ng nổ của c#244;ng nghệ, thị trường n#224;y kh#244;ng muốn giảm”, một nh#224; quản l#253; quỹ n#243;i...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 09:50:00 +0700</t>
+          <t>Tue, 12 May 2026 01:19:45 GMT</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://cafef.vn/chu-tich-doan-nguyen-duc-gom-them-co-phieu-hag-188260513092755881.chn</t>
+          <t>https://vneconomy.vn/chung-khoan-my-van-lap-dinh-moi-du-dam-phan-hoa-binh-be-tac-gia-dau-tang-3.htm</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dabaco chia cổ tức tổng tỷ lệ 15%</t>
+          <t>Thị trường đang thử thách quyết tâm bảo vệ tỷ giá đồng yên của Nhật Bản</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dabaco sẽ trả cổ tức 3% bằng tiền, tức 300 đồng/cổ phiếu và 12% bằng cổ phiếu. Dự kiến thực hiện trong quý II/2026.</t>
+          <t>Bởi vậy, nếu BOJ tiếp tục giữ nguy#234;n thay v#236; tăng l#227;i suất, xu hướng mất gi#225; của đồng y#234;n c#243; thể c#242;n tiếp tục...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 09:31:00 +0700</t>
+          <t>Tue, 12 May 2026 00:02:03 GMT</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://cafef.vn/dabaco-chia-co-tuc-tong-ty-le-15-188260513092502696.chn</t>
+          <t>https://vneconomy.vn/thi-truong-dang-thu-thach-quyet-tam-bao-ve-ty-gia-dong-yen-cua-nhat-ban.htm</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Vinhomes phát hành liên tiếp 2 lô trái phiếu trị giá 3.000 tỷ đồng</t>
+          <t>FiinGroup: Áp lực biên lợi nhuận khiến các ngân hàng khó giảm lãi suất ngay trong ngắn hạn</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ngày 11/5 vừa qua, Vinhomes đã phát hành liên tiếp 02 lô trái phiếu trong cùng ngày 11/5/2026 với tổng giá trị huy động 3.000 tỷ đồng.</t>
+          <t>Theo Fiingroup l#227;i suất cho vay được dự b#225;o sẽ kh#243; giảm ngay trong ngắn hạn khi bi#234;n lợi nhuận của c#225;c ng#226;n h#224;ng đang chịu #225;p lực thu hẹp r#245; rệt.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 09:29:00 +0700</t>
+          <t>Tue, 12 May 2026 00:01:27 GMT</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://cafef.vn/vinhomes-phat-hanh-lien-tiep-2-lo-trai-phieu-tri-gia-3000-ty-dong-188260513092558919.chn</t>
+          <t>https://vneconomy.vn/fiingroup-ap-luc-bien-loi-nhuan-khien-cac-ngan-hang-kho-giam-lai-suat-ngay-trong-ngan-han.htm</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nhiều lãnh đạo Imexpharm bán cổ phiếu trong cùng một phiên</t>
+          <t>Lãi suất tiết kiệm ngân hàng nào cao nhất?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tổng giám đốc Trần Thị Đào cùng 2 Phó Tổng giám đốc và Kế toán trưởng Imexpharm đồng loạt bán cổ phiếu IMP trong cùng một phiên.</t>
+          <t>Lãi suất tiết kiệm hạ nhiệt sau chỉ đạo của Thống đốc song mặt bằng chung với các khoản thỏa thuận vẫn ở mức hấp dẫn, một số nhà băng trả 8-9% một năm.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 08:17:00 +0700</t>
+          <t>Tue, 12 May 2026 05:33:34 +0700</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://cafef.vn/nhieu-lanh-dao-imexpharm-ban-co-phieu-trong-cung-mot-phien-188260513072238693.chn</t>
+          <t>https://vnexpress.net/lai-suat-tiet-kiem-ngan-hang-nao-cao-nhat-5072646.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Vì sao nhà đầu tư 'chưa về bờ' dù VN-Index vượt đỉnh?</t>
+          <t>Tháng 4, HNX huy động 45.455 tỷ đồng qua đấu thầu trái phiếu Chính phủ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nhiều nhà đầu tư vẫn đang lỗ vài chục phần trăm vì danh mục tập trung vào chứng khoán, công nghệ, dầu khí mà không có cổ phiếu họ Vingroup.</t>
+          <t>T#237;nh lũy kế từ đầu năm, Kho bạc Nh#224; nước đ#227; huy động được 125.556 tỷ đồng, ho#224;n th#224;nh 41% kế hoạch ph#225;t h#224;nh qu#253; 2 v#224; đạt 25% kế hoạch ph#225;t h#224;nh của năm 2026.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 06:08:00 +0700</t>
+          <t>Mon, 11 May 2026 12:47:52 GMT</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/vi-sao-nha-dau-tu-chua-ve-bo-du-vn-index-vuot-dinh-5072532.html</t>
+          <t>https://vneconomy.vn/thang-4-hnx-huy-dong-45455-ty-dong-qua-dau-thau-trai-phieu-chinh-phu.htm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SACOMBANK lập kỷ lục: Từ “bàn tay vàng” của ông Nguyễn Đức Thuỵ đến pha đổi tên đậm chất “phong thuỷ”</t>
+          <t>Australia khởi xướng điều tra đối với thép mạ kẽm nhập khẩu từ Việt Nam</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sự xuất hiện của ông Nguyễn Đức Thuỵ tại SACOMBANK từ cuối năm 2025 kéo theo hàng loạt thay đổi mang tính chiến lược đối với ngân hàng.</t>
+          <t>Australia vừa ch#237;nh thức khởi xướng điều tra đối với sản phẩm th#233;p mạ kẽm nhập khẩu từ Việt Nam. D#249; đối mặt với c#225;o buộc bi#234;n độ ph#225; gi#225; ở mức cao, c#225;c doanh nghiệp trong nước vẫn tự tin v#224;o khả năng bảo vệ lợi #237;ch hợp ph#225;p dựa tr#234;n số liệu thực tế v#224; kinh nghiệm d#224;y dạn...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 00:10:00 +0700</t>
+          <t>Mon, 11 May 2026 09:53:09 GMT</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://cafef.vn/sacombank-lap-ky-luc-tu-ban-tay-vang-cua-ong-nguyen-duc-thuy-den-pha-doi-ten-dam-chat-phong-thuy-188260512232819282.chn</t>
+          <t>https://vneconomy.vn/australia-khoi-xuong-dieu-tra-doi-voi-thep-ma-kem-nhap-khau-tu-viet-nam.htm</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Thêm công ty chứng khoán hạ dự phóng VN-Index năm 2026</t>
+          <t>Giá vàng lao dốc sau khi Mỹ từ chối đề xuất phản hồi của Iran</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CTCK này cho rằng nền tảng vĩ mô ổn định, triển vọng tăng trưởng lợi nhuận tích cực và định giá còn tương đối hấp dẫn vẫn là cơ sở để VN-Index duy trì xu hướng tăng trong năm 2026.</t>
+          <t>Gi#225; v#224;ng thế giới giảm mạnh v#224;o đầu giờ phi#234;n s#225;ng nay (11/5) tại thị trường ch#226;u #193;, sau khi c#243; tin Mỹ từ chối đề xuất m#224; Iran đưa ra để phản hồi kế hoạch h#242;a b#236;nh của Mỹ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 00:08:00 +0700</t>
+          <t>Mon, 11 May 2026 00:44:18 GMT</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://cafef.vn/them-cong-ty-chung-khoan-ha-du-phong-vn-index-nam-2026-188260512213008592.chn</t>
+          <t>https://vneconomy.vn/gia-vang-lao-doc-sau-khi-my-tu-choi-de-xuat-phan-hoi-cua-iran.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gần 7 triệu cổ phiếu sang tay, STB lập đỉnh</t>
+          <t>Giá vàng tuần này có thể tăng</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sau pha điều chỉnh ở phiên trước, thị trường chứng khoán hôm nay (12/5) hồi phục trở lại khi VN-Index lấy lại mốc 1.900 điểm. Dòng tiền tập trung vào nhóm ngân hàng và dầu khí, trong đó STB trở thành tâm điểm với mức tăng cận trần, lập đỉnh giá lịch sử mới.</t>
+          <t>Tiếp đà phục hồi tuần qua, Phố Wall lẫn nhà đầu tư cá nhân cùng dự báo giá vàng tăng, với kỳ vọng hạ nhiệt căng thẳng Mỹ - Iran.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 18:24:00 +0700</t>
+          <t>Mon, 11 May 2026 00:00:00 +0700</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://cafef.vn/gan-7-trieu-co-phieu-sang-tay-stb-lap-dinh-188260512174905008.chn</t>
+          <t>https://vnexpress.net/gia-vang-tuan-nay-co-the-tang-5072198.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VN-Index trở lại mốc 1.900 điểm, dòng tiền tìm đến cổ phiếu bất động sản</t>
+          <t>Dấu ấn kinh tế thế giới tuần 2-9/5/2026: Đồn đoán về Nhật Bản can thiệp tỷ giá, Mỹ chờ câu trả lời từ Iran</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Thị trường chứng khoán ngày 12-5 ghi nhận nhịp hồi phục đáng chú ý khi VN-Index lấy lại mốc 1.900 điểm sau phiên rung lắc mạnh đầu ngày</t>
+          <t>Trong tuần n#224;y, thị trường t#224;i ch#237;nh to#224;n cầu tin rằng nh#224; chức tr#225;ch Nhật Bản đ#227; c#243; đợt can thiệp thứ hai v#224;o thị trường ngoại hối để bảo vệ tỷ gi#225; đồng y#234;n...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 17:52:00 +0700</t>
+          <t>Sun, 10 May 2026 00:34:52 GMT</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://cafef.vn/vn-index-tro-lai-moc-1900-diem-dong-tien-tim-den-co-phieu-bat-dong-san-188260512175253.chn</t>
+          <t>https://vneconomy.vn/dau-an-kinh-te-the-gioi-tuan-2-952026-don-doan-ve-nhat-ban-can-thiep-ty-gia-my-cho-cau-tra-loi-tu-iran.htm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cổ phiếu Sacombank (STB) tăng cận trần sau biến động nhân sự cấp cao</t>
+          <t>MSCI và FTSE khác nhau thế nào trong nâng hạng thị trường chứng khoán?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cổ phiếu STB của Sacombank bất ngờ trở thành tâm điểm hút dòng tiền từ các nhà đầu tư trong phiên 12/5, khi tăng cận trần – lập đỉnh giá lịch sử mới ngay sau thông tin ngân hàng bổ nhiệm nhân sự cấp cao.</t>
+          <t>Cùng là nâng hạng thị trường chứng khoán, nhưng MSCI và FTSE có tiêu chí, tầm ảnh hưởng và sức hấp dẫn khác nhau.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 16:44:00 +0700</t>
+          <t>Sun, 10 May 2026 00:02:00 +0700</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://cafef.vn/co-phieu-sacombank-stb-tang-can-tran-sau-bien-dong-nhan-su-cap-cao-188260512160131532.chn</t>
+          <t>https://vnexpress.net/msci-va-ftse-khac-nhau-the-nao-trong-nang-hang-thi-truong-chung-khoan-5070886.html</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>VN-Index quay lại mốc 1.900 điểm</t>
+          <t>SP 500 đóng cửa cao kỷ lục sau báo cáo việc làm, giá dầu chững lại</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bất chấp hai cổ phiếu "họ" Vingroup tiếp tục giảm, VN-Index vẫn tăng hơn 5 điểm, lên 1.901 điểm nhờ trạng thái hưng phấn của nhóm dầu khí và một số mã ngân hàng.</t>
+          <t>Thị trường chứng kho#225;n Mỹ tăng điểm trong phi#234;n giao dịch ng#224;y thứ S#225;u (8/5), khi số liệu việc l#224;m khả quan hơn dự b#225;o mang lại cho nh#224; đầu tư sự y#234;n t#226;m về sức khỏe của nền kinh tế...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 16:10:36 +0700</t>
+          <t>Sat, 09 May 2026 01:12:23 GMT</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/vn-index-quay-lai-moc-1-900-diem-5073096.html</t>
+          <t>https://vneconomy.vn/sp-500-dong-cua-cao-ky-luc-sau-bao-cao-viec-lam-gia-dau-chung-lai.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Phiên 12/5: Khối ngoại vẫn bán ròng hơn 800 tỷ đồng, cổ phiếu nào bị "xả" mạnh nhất?</t>
+          <t>CEO Nvidia, Apple sẽ cùng ông Trump đến Trung Quốc</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Chiều mua, khối ngoại mua ròng mạnh nhất cổ phiếu VIC với giá trị 196 tỷ đồng, xếp sau là VRE với 118 tỷ đồng.</t>
+          <t>Hơn 10 lãnh đạo doanh nghiệp, trong đó có CEO Nvidia, Apple, Qualcomm, Citigroup và Boeing sẽ cùng Tổng thống Mỹ đến Trung Quốc tuần tới.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 15:45:00 +0700</t>
+          <t>Sat, 09 May 2026 00:00:00 +0700</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://cafef.vn/phien-12-5-khoi-ngoai-van-ban-rong-hon-800-ty-dong-co-phieu-nao-bi-xa-manh-nhat-188260512151657978.chn</t>
+          <t>https://vnexpress.net/ceo-nvidia-apple-se-cung-ong-trump-den-trung-quoc-5071620.html</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PVTrans sắp phát hành gần 47 triệu cổ phiếu trả cổ tức</t>
+          <t>Thủ tướng Sri Lanka muốn doanh nghiệp Việt tăng hợp tác thương mại, hàng không</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PVTrans lên kế hoạch phát hành gần 47 triệu cổ phiếu trả cổ tức cho cổ đông với tỷ lệ thực hiện quyền 100:10. Nếu thành công, vốn điều lệ của doanh nghiệp sẽ lên mức 5.169 tỷ đồng.</t>
+          <t>Thủ tướng Sri Lanka muốn doanh nghiệp Việt mở rộng hợp tác trong lĩnh vực thương mại, chế biến thực phẩm, logistics, hàng không và du lịch.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 14:40:00 +0700</t>
+          <t>Fri, 08 May 2026 21:48:02 +0700</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://cafef.vn/pvtrans-sap-phat-hanh-gan-47-trieu-co-phieu-tra-co-tuc-18826051214334115.chn</t>
+          <t>https://vnexpress.net/thu-tuong-sri-lanka-muon-doanh-nghiep-viet-tang-hop-tac-thuong-mai-hang-khong-5071709.html</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SJC lãi kỷ lục dù doanh thu thấp nhất 10 năm</t>
+          <t>Chủ tịch UBCKNN chỉ ra yếu tố "sống còn" để chứng khoán Việt Nam thu hút dòng vốn ngoại</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doanh thu ở mức thấp nhất một thập kỷ, Công ty SJC vẫn có lợi nhuận sau thuế tăng 9% lên mức kỷ lục 425,5 tỷ đồng năm ngoái.</t>
+          <t>Theo lãnh đạo UBCKNN, việc minh bạch hóa thông tin và huy động vốn thông qua thị trường quốc tế là yếu tố rất quan trọng, đặc biệt trong việc thu hút các nhà đầu tư tổ chức và nhà đầu tư nước ngoài có xu hướng gắn bó dài hạn với doanh nghiệp</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 12:13:58 +0700</t>
+          <t>Thu, 14 May 26 09:42:00 +0700</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/sjc-lai-ky-luc-du-doanh-thu-thap-nhat-10-nam-5072912.html</t>
+          <t>https://cafef.vn/chu-tich-ubcknn-chi-ra-yeu-to-song-con-de-chung-khoan-viet-nam-thu-hut-dong-von-ngoai-188260514094307668.chn</t>
         </is>
       </c>
     </row>
@@ -1218,17 +1218,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Chứng khoán VietinBank sắp phát hành 59,5 triệu cổ phiếu trả cổ tức</t>
+          <t>Dẫn đầu danh sách chậm đóng bảo hiểm TP.HCM, Xây dựng Hòa Bình đang làm ăn ra sao?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Chứng khoán VietinBank dự kiến phát hành 59,55 triệu cổ phiếu trả cổ tức, tương ứng tỷ lệ thực hiện quyền 100:28.</t>
+          <t>Dù ghi nhận lợi nhuận quý I/2026 tăng gấp hơn 4 lần so với cùng kỳ, Xây dựng Hòa Bình vẫn tiếp tục dẫn đầu danh sách chậm đóng bảo hiểm TP.HCM với số tiền gần 71,1 tỷ đồng.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 11:39:00 +0700</t>
+          <t>Thu, 14 May 26 08:10:00 +0700</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://cafef.vn/chung-khoan-vietinbank-sap-phat-hanh-595-trieu-co-phieu-tra-co-tuc-18826051210395094.chn</t>
+          <t>https://cafef.vn/dan-dau-danh-sach-cham-dong-bao-hiem-tphcm-xay-dung-hoa-binh-dang-lam-an-ra-sao-188260514081107854.chn</t>
         </is>
       </c>
     </row>
@@ -1248,17 +1248,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Xu hướng chủ đạo vẫn là tăng trưởng, chuyên gia tiết lộ “mỏ vàng” trên sàn chứng khoán</t>
+          <t>Phó Giám đốc SSI Research chỉ ra hai cổ phiếu bán lẻ "sáng cửa" nhờ câu chuyện IPO khủng và định giá hấp dẫn</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Theo chuyên gia AAS, việc mua được “hàng tốt” ở “mức giá thấp” là lợi thế lớn nhất để có biên lợi nhuận vượt trội trong tương lai.</t>
+          <t>Mặc dù triển vọng dài hạn của ngành bán lẻ vẫn rất khả quan với định giá P/E dự phóng thấp hơn trung bình 5 năm, song chuyên gia cho rằng nhà đầu tư ngắn hạn cần giữ thái độ thận trọng.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 11:18:00 +0700</t>
+          <t>Thu, 14 May 26 00:03:00 +0700</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1266,29 +1266,29 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://cafef.vn/xu-huong-chu-dao-van-la-tang-truong-chuyen-gia-tiet-lo-mo-vang-tren-san-chung-khoan-18826051211180719.chn</t>
+          <t>https://cafef.vn/pho-giam-doc-ssi-research-chi-ra-hai-co-phieu-ban-le-sang-cua-nho-cau-chuyen-ipo-khung-va-dinh-gia-hap-dan-188260513222817243.chn</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MSR đạt doanh thu gần 3.000 tỷ trong quý I</t>
+          <t>Một doanh nghiệp cao su bất ngờ tăng trần 5 phiên, HOSE yêu cầu giải trình</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Doanh thu Masan High-Tech Materials (MSR) tăng gần 115% so với cùng kỳ, đạt 2.993 tỷ trong quý I/2026 nhờ sự cải thiện đồng thời của giá hàng hóa, sản lượng và cấu trúc tài chính.</t>
+          <t>Trong 5 phiên liên tiếp từ 07-13/05/2026, cổ phiếu HRC của CTCP Cao su Hòa Bình (Horuco) đều tím trần. Với diễn biến này, Sở Giao dịch Chứng khoán TP.HCM (HOSE) đã có văn bản yêu cầu Horuco giải trình.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 09:00:00 +0700</t>
+          <t>Wed, 13 May 2026 19:17:24 +0700</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1296,29 +1296,29 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/msr-dat-doanh-thu-gan-3-000-ty-trong-quy-i-5072256.html</t>
+          <t>http://vietstock.vn/2026/05/mot-doanh-nghiep-cao-su-bat-ngo-tang-tran-5-phien-hose-yeu-cau-giai-trinh-830-1442288.htm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Chuỗi nhà thuốc của Thế Giới Di Động sắp hết lỗ</t>
+          <t>MSR bán thành công 2% cổ phần, đáp ứng điều kiện công ty đại chúng</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thế Giới Di Động cho biết chuỗi nhà thuốc An Khang "gần ngưỡng hòa vốn" và có thể đóng góp lợi nhuận sau khoảng 8 năm doanh nghiệp này tham gia mảng bán lẻ dược.</t>
+          <t>Ngày 13/05/2026, CTCP Tập đoàn Masan (HOSE: MSN) công bố công ty con mà Masan sở hữu 100% vốn đã hoàn tất việc bán 21.99 triệu cp, tương đương 2% tổng số cổ phiếu đang lưu hành của CTCP Masan High-Tech Materials (UPCoM: MSR), thông qua các giao dịch trên hệ thống UPCoM theo đúng quy định hiện hành.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 00:02:00 +0700</t>
+          <t>Wed, 13 May 2026 17:37:35 +0700</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1326,29 +1326,29 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/chuoi-nha-thuoc-cua-the-gioi-di-dong-sap-het-lo-5072234.html</t>
+          <t>http://vietstock.vn/2026/05/msr-ban-thanh-cong-2-co-phan-dap-ung-dieu-kien-cong-ty-dai-chung-830-1442192.htm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>VN-Index lên 1.915 điểm</t>
+          <t>IDJ ký hợp đồng kiểm toán mới kỳ vọng khắc phục tình trạng cổ phiếu bị cảnh báo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dù hơn 58% mã giảm giá, chứng khoán vẫn đóng cửa ở mức cao kỷ lục 1.915 điểm nhờ sự hỗ trợ của cổ phiếu nhóm Vingroup và ngân hàng.</t>
+          <t>CTCP IDJ Việt Nam (HNX: IDJ) vừa báo cáo cơ quan quản lý về các biện pháp và lộ trình khắc phục tình trạng cổ phiếu bị cảnh báo, với trọng tâm là việc ký hợp đồng kiểm toán Báo cáo tài chính năm 2025 với Công ty TNHH Kiểm toán và Tư vấn UHY (UHY). Công ty cho biết sẽ thực hiện việc Công bố Báo cáo tài chính 2025 đã được kiểm toán đúng theo các quy định của pháp luật để sớm đưa cổ phiếu ra khỏi diện bị cảnh báo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 15:54:08 +0700</t>
+          <t>Wed, 13 May 2026 17:12:43 +0700</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1356,29 +1356,29 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/vn-index-len-1-915-diem-5071587.html</t>
+          <t>http://vietstock.vn/2026/05/idj-ky-hop-dong-kiem-toan-moi-ky-vong-khac-phuc-tinh-trang-co-phieu-bi-canh-bao-830-1442032.htm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cổ phiếu PC1 giảm mạnh</t>
+          <t>Gelex Electric tăng vốn điều lệ vượt 6.400 tỷ đồng sau đợt phát hành cổ phiếu thưởng</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cổ phiếu PC1 chạm giá sàn và chốt phiên giảm 5% với thanh khoản lớn.</t>
+          <t>Kết thúc đợt phát hành ngày 6/5/2026, Gelex Electric đã phân phối thành công gần 274,5 triệu cổ phiếu cho 5.060 cổ đông, qua đó tăng vốn điều lệ lên mức gần 6.405 tỷ đồng.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 15:21:50 +0700</t>
+          <t>Wed, 13 May 26 17:09:00 +0700</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1386,29 +1386,29 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/co-phieu-pc1-giam-manh-5071548.html</t>
+          <t>https://cafef.vn/gelex-electric-tang-von-dieu-le-vuot-6400-ty-dong-sau-dot-phat-hanh-co-phieu-thuong-188260513164543308.chn</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CEO Hóa chất Đức Giang: Sẽ kế thừa ý chí, tầm nhìn của ông Đào Hữu Huyền</t>
+          <t>Công bố giá xăng E10 Petrolimex</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ông Lưu Bách Đạt, Tổng giám đốc Hóa chất Đức Giang, hứa dàn lãnh đạo mới sẽ vận hành tốt doanh nghiệp, kế thừa ý chí, tầm nhìn của cựu Chủ tịch Đào Hữu Huyền.</t>
+          <t>Tập đoàn Xăng dầu Việt Nam (Petrolimex) vừa thông báo giá bán xăng sinh học E10 RON 95 áp dụng từ ngày 0h ngày 13/5. Theo đó, giá bán xăng sinh học E10 RON 95-V tại cửa hàng xăng dầu tại thị trường vùng 1 là 24.630 đồng/lít, tại các thị trường vùng 2 là 25.120 đồng/lít.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Fri, 08 May 2026 13:09:09 +0700</t>
+          <t>Wed, 13 May 26 16:45:00 +0700</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1416,157 +1416,157 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/ceo-hoa-chat-duc-giang-se-ke-thua-y-chi-tam-nhin-cua-ong-dao-huu-huyen-5071498.html</t>
+          <t>https://cafef.vn/cong-bo-gia-xang-e10-petrolimex-188260513154754794.chn</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Một doanh nghiệp đầu ngành sắp lăn chốt cổ tức tiền mặt 83%, "đại gia" Thái Lan vớ bẫm</t>
+          <t>Cổ phiếu dầu khí hút tiền nhà đầu tư trong nước</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Đây cũng là mức cổ tức tiền mặt cao nhất trong lịch sử hoạt động của doanh nghiệp.</t>
+          <t>Toàn bộ cổ phiếu dầu khí bật mạnh, trong đó GAS chạm trần và dẫn đầu danh sách "trụ đỡ" của VN-Index trước áp lực xả hàng cổ phiếu Vingroup.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 16:11:00 +0700</t>
+          <t>Wed, 13 May 2026 16:25:11 +0700</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://cafef.vn/mot-doanh-nghiep-dau-nganh-sap-lan-chot-co-tuc-tien-mat-83-dai-gia-thai-lan-vo-bam-188260513161023867.chn</t>
+          <t>https://vnexpress.net/co-phieu-dau-khi-hut-tien-nha-dau-tu-trong-nuoc-5073515.html</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>​Chuyên gia quốc tế: Việt Nam có cơ hội thành 'tọa độ vàng' siêu sự kiện</t>
+          <t>Chứng khoán 13-5: Điều gì khiến cổ phiếu dầu khí bùng nổ?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Chính sách mở đường và làn sóng đầu tư hạ tầng quy mô lớn đang tạo đà cho nền công nghiệp văn hóa Việt Nam bứt phá, vươn tầm thành điểm đến mới của kinh tế trải nghiệm toàn cầu.</t>
+          <t>Phiên giao dịch ngày 13-5 ghi nhận diễn biến đầy biến động của thị trường chứng khoán khi áp lực bán mạnh xuất hiện ở nhóm cổ phiếu vốn hóa lớn</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 16:00:00 +0700</t>
+          <t>Wed, 13 May 26 16:14:00 +0700</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/chuyen-gia-quoc-te-viet-nam-co-co-hoi-thanh-toa-do-vang-sieu-su-kien-5073499.html</t>
+          <t>https://cafef.vn/chung-khoan-13-5-dieu-gi-khien-co-phieu-dau-khi-bung-no-18826051316143265.chn</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fecon sắp phát hành lô trái phiếu 125 tỷ đồng</t>
+          <t>SSIAM - CCIX và Daiwa ký kết hợp tác, mở rộng đầu tư vốn Nhật Bản vào Việt Nam</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Fecon dự kiến phát hành 1.250 trái phiếu mã FCN12601 ra thị trường trong nước vào ngày 15/5/2026, mệnh giá 100 triệu đồng/trái phiếu, qua đó huy động 125 tỷ đồng.</t>
+          <t>SSI, CCI CrossBorder (CCIX) v#224; Daiwa Corporate Investment (DCI) vừa k#253; kết Thỏa thuận hợp tác nhằm thiết lập khu#244;n khổ hợp t#225;c chiến lược, hướng tới tạo lập v#224; mở rộng c#225;c cơ hội đồng đầu tư v#224; k#234;́t n#244;́i t#224;i trợ vốn giữa các định ch#234;́ tài chính Nhật Bản với c#225;c doanh nghiệp Việt Nam.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 15:50:00 +0700</t>
+          <t>Wed, 13 May 2026 07:44:52 GMT</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://cafef.vn/fecon-sap-phat-hanh-lo-trai-phieu-125-ty-dong-188260513144942479.chn</t>
+          <t>https://vneconomy.vn/ssiam-ccix-va-daiwa-ky-ket-hop-tac-mo-rong-dau-tu-von-nhat-ban-vao-viet-nam.htm</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ngân hàng tiếp tục rao bán nhà máy nông sản hơn 1.200 tỷ liên quan bà Trương Mỹ Lan</t>
+          <t>SSIAM bắt tay 2 định chế tài chính, mở rộng cơ hội đầu tư và tài trợ vốn giữa Nhật Bản và Việt Nam</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>VietinBank phát mãi lần hai nhà máy Tanifood Tây Ninh liên quan vụ án Vạn Thịnh Phát với giá khởi điểm 1.200 tỷ đồng, thấp hơn 10% so với lần rao bán trước.</t>
+          <t>Phát huy chuyên môn, mạng lưới và nguồn lực của từng bên, SSIAM, CCIX và DCI sẽ chủ động tìm kiếm, cấu trúc và triển khai các cơ hội đầu tư và tài trợ vốn trung, dài hạn, góp phần thúc đẩy tăng trưởng bền vững cho doanh nghiệp Việt Nam và nền kinh tế.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 15:47:20 +0700</t>
+          <t>Wed, 13 May 26 13:53:00 +0700</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/ngan-hang-tiep-tuc-rao-ban-nha-may-nong-san-hon-1-200-ty-lien-quan-ba-truong-my-lan-5073438.html</t>
+          <t>https://cafef.vn/ssiam-bat-tay-2-dinh-che-tai-chinh-mo-rong-co-hoi-dau-tu-va-tai-tro-von-giua-nhat-ban-va-viet-nam-188260513135311114.chn</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Phiên 13/5: Khối ngoại tiếp đà bán ròng nghìn tỷ, ngược chiều gom mạnh một cổ phiếu ngân hàng</t>
+          <t>Cổ phiếu dầu khí phục hồi mạnh, GAS kịch trần</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Giao dịch của khối ngoại là điểm trừ khi bán ròng khoảng 1.475 tỷ đồng.</t>
+          <t>Sự yếu ớt của nh#243;m cổ phiếu dẫn dắt tiếp tục g#226;y sức #233;p l#234;n VN-Index s#225;ng nay d#249; độ rộng chỉ số kh#244;ng thực sự k#233;m. Mức độ ph#226;n h#243;a v#224; ổn định ở chỉ số tạo điều kiện cho d#242;ng tiền ngắn hạn hoạt động mạnh hơn, đặc biệt nh#243;m dầu kh#237; đang phục hồi kh#225; ấn tượng.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 15:45:00 +0700</t>
+          <t>Wed, 13 May 2026 05:03:42 GMT</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://cafef.vn/phien-13-5-khoi-ngoai-tiep-da-ban-rong-nghin-ty-nguoc-chieu-gom-manh-mot-co-phieu-ngan-hang-1882605131542172.chn</t>
+          <t>https://vneconomy.vn/co-phieu-dau-khi-phuc-hoi-manh-gas-kich-tran.htm</t>
         </is>
       </c>
     </row>
@@ -1578,25 +1578,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Vừa về tay ông lớn dược phẩm Trung Quốc, loạt lãnh đạo Imexpharm cùng bán ra lượng cổ phiếu</t>
+          <t>FPT báo lãi tháng 4/2026 tăng 21%</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Nhiều lãnh đạo của Công ty cổ phần Dược phẩm Imexpharm (MCK: IMP, sàn: HoSE) vừa báo cáo kết quả bán ra cổ phiếu.</t>
+          <t>FPT cho biết khối lượng đơn hàng ký mới tại thị trường nước ngoài đã tăng vọt 30% so với cùng kỳ.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 15:20:00 +0700</t>
+          <t>Wed, 13 May 26 12:03:00 +0700</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://cafef.vn/vua-ve-tay-ong-lon-duoc-pham-trung-quoc-loat-lanh-dao-imexpharm-cung-ban-ra-luong-co-phieu-188260513145031724.chn</t>
+          <t>https://cafef.vn/fpt-bao-lai-thang-4-2026-tang-21-188260513120329893.chn</t>
         </is>
       </c>
     </row>
@@ -1608,25 +1608,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Người nhà lãnh đạo SeABank đăng ký mua 5 triệu cổ phiếu SSB</t>
+          <t>Chủ tịch Đoàn Nguyên Đức gom thêm cổ phiếu HAG</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ông Lê Hữu Báu, chồng của bà Nguyễn Thị Nga- Phó Chủ tịch thường trực HĐQT SeABank, vừa đăng ký mua 5 triệu cổ phiếu SSB nhằm mục đích tăng tỷ lệ sở hữu.</t>
+          <t>Ông Đoàn Nguyên Đức- Chủ tịch HĐQT Hoàng Anh Gia Lai, đã mua vào 4 triệu cổ phiếu HAG bằng phương thức khớp lệnh trên sàn, qua đó nâng sở hữu lên 25,09%.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 15:18:00 +0700</t>
+          <t>Wed, 13 May 26 09:50:00 +0700</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://cafef.vn/nguoi-nha-lanh-dao-seabank-dang-ky-mua-5-trieu-co-phieu-ssb-188260513145128351.chn</t>
+          <t>https://cafef.vn/chu-tich-doan-nguyen-duc-gom-them-co-phieu-hag-188260513092755881.chn</t>
         </is>
       </c>
     </row>
@@ -1638,175 +1638,175 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Một doanh nghiệp “lạ” trả cổ tức kỷ lục 60% bằng tiền mặt</t>
+          <t>Dabaco chia cổ tức tổng tỷ lệ 15%</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Đây là công ty duy nhất trên sàn bán các loại kềm.</t>
+          <t>Dabaco sẽ trả cổ tức 3% bằng tiền, tức 300 đồng/cổ phiếu và 12% bằng cổ phiếu. Dự kiến thực hiện trong quý II/2026.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 14:41:00 +0700</t>
+          <t>Wed, 13 May 26 09:31:00 +0700</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://cafef.vn/mot-doanh-nghiep-la-tra-co-tuc-ky-luc-60-bang-tien-mat-18826051314410115.chn</t>
+          <t>https://cafef.vn/dabaco-chia-co-tuc-tong-ty-le-15-188260513092502696.chn</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Phát hiện giá Bitcoin tương quan với thị trường cá cược thể thao</t>
+          <t>Vinhomes phát hành liên tiếp 2 lô trái phiếu trị giá 3.000 tỷ đồng</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Diễn biến giá của Bitcoin và quỹ ETF lớn nhất thế giới về cá cược thể thao có mối liên hệ về mặt thống kê tới hơn 80%.</t>
+          <t>Ngày 11/5 vừa qua, Vinhomes đã phát hành liên tiếp 02 lô trái phiếu trong cùng ngày 11/5/2026 với tổng giá trị huy động 3.000 tỷ đồng.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 14:35:54 +0700</t>
+          <t>Wed, 13 May 26 09:29:00 +0700</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/phat-hien-gia-bitcoin-tuong-quan-voi-thi-truong-ca-cuoc-the-thao-5073356.html</t>
+          <t>https://cafef.vn/vinhomes-phat-hanh-lien-tiep-2-lo-trai-phieu-tri-gia-3000-ty-dong-188260513092558919.chn</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Agribank thúc đẩy giải pháp ngân hàng số khu vực Tây Nam Bộ</t>
+          <t>Ngại rủi ro, quỹ SGI Capital duy trì tiền mặt cao hơn 70%</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Agribank đẩy mạnh các giải pháp thanh toán không tiền mặt, mở rộng hạ tầng giao dịch, thúc đẩy tài chính số khu vực nông thôn Tây Nam Bộ.</t>
+          <t>SGI Capital tiếp tục giữ tỷ trọng tiền mặt cao l#234;n 70,49%, c#242;n lại l#224; ph#226;n bổ v#224;o danh mục c#225;c cổ phiếu gồm DRI, VIP, FMC, BWE, TLG, FPT, ACB, SIP, MWG.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 14:00:00 +0700</t>
+          <t>Wed, 13 May 2026 02:07:49 GMT</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/agribank-thuc-day-giai-phap-ngan-hang-so-khu-vuc-tay-nam-bo-5073401.html</t>
+          <t>https://vneconomy.vn/ngai-rui-ro-quy-sgi-capital-duy-tri-tien-mat-cao-hon-70.htm</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>VinFast sẽ tách mảng sản xuất tại Việt Nam</t>
+          <t>Nhiều lãnh đạo Imexpharm bán cổ phiếu trong cùng một phiên</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>VinFast dự kiến chuyển giao mảng sản xuất cho nhóm nhà đầu tư mới với giá khoảng 530 triệu USD và ông Phạm Nhật Vượng vẫn tham gia pháp nhân mới nhưng giảm tỷ lệ sở hữu.</t>
+          <t>Tổng giám đốc Trần Thị Đào cùng 2 Phó Tổng giám đốc và Kế toán trưởng Imexpharm đồng loạt bán cổ phiếu IMP trong cùng một phiên.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 10:46:42 +0700</t>
+          <t>Wed, 13 May 26 08:17:00 +0700</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/vinfast-se-tach-mang-san-xuat-tai-viet-nam-5073349.html</t>
+          <t>https://cafef.vn/nhieu-lanh-dao-imexpharm-ban-co-phieu-trong-cung-mot-phien-188260513072238693.chn</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bà Huỳnh Bích Ngọc muốn bán 15 triệu cổ phiếu AgriS</t>
+          <t>Vì sao nhà đầu tư 'chưa về bờ' dù VN-Index vượt đỉnh?</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bà Huỳnh Bích Ngọc đăng ký bán ra 15 triệu cổ phiếu SBT của AgriS nhằm mục đích cơ cấu danh mục đầu tư.</t>
+          <t>Nhiều nhà đầu tư vẫn đang lỗ vài chục phần trăm vì danh mục tập trung vào chứng khoán, công nghệ, dầu khí mà không có cổ phiếu họ Vingroup.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 09:34:00 +0700</t>
+          <t>Wed, 13 May 2026 06:08:00 +0700</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://cafef.vn/ba-huynh-bich-ngoc-muon-ban-15-trieu-co-phieu-agris-188260513092914186.chn</t>
+          <t>https://vnexpress.net/vi-sao-nha-dau-tu-chua-ve-bo-du-vn-index-vuot-dinh-5072532.html</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Giới đầu tư kỳ vọng gì vào thượng đỉnh Mỹ - Trung?</t>
+          <t>SACOMBANK lập kỷ lục: Từ “bàn tay vàng” của ông Nguyễn Đức Thuỵ đến pha đổi tên đậm chất “phong thuỷ”</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Giới đầu tư dự báo khó có thỏa thuận kinh tế đột phá, dồn chú ý vào diễn biến lĩnh vực AI tại cuộc gặp lãnh đạo Mỹ - Trung.</t>
+          <t>Sự xuất hiện của ông Nguyễn Đức Thuỵ tại SACOMBANK từ cuối năm 2025 kéo theo hàng loạt thay đổi mang tính chiến lược đối với ngân hàng.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Wed, 13 May 2026 00:08:00 +0700</t>
+          <t>Wed, 13 May 26 00:10:00 +0700</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/gioi-dau-tu-ky-vong-gi-vao-thuong-dinh-my-trung-5073144.html</t>
+          <t>https://cafef.vn/sacombank-lap-ky-luc-tu-ban-tay-vang-cua-ong-nguyen-duc-thuy-den-pha-doi-ten-dam-chat-phong-thuy-188260512232819282.chn</t>
         </is>
       </c>
     </row>
@@ -1818,55 +1818,55 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tiền lớn chọn lọc, chuyên gia chỉ tên nhóm cổ phiếu xếp hạng cao trên thị trường</t>
+          <t>Thêm công ty chứng khoán hạ dự phóng VN-Index năm 2026</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Trong bối cảnh dòng tiền tiếp tục ưu tiên các cổ phiếu có sức mạnh vượt trội, chuyên gia ABS đã tiến hành lọc ra các nhóm ngành và cổ phiếu có mức độ mạnh nhất so với thị trường chung.</t>
+          <t>CTCK này cho rằng nền tảng vĩ mô ổn định, triển vọng tăng trưởng lợi nhuận tích cực và định giá còn tương đối hấp dẫn vẫn là cơ sở để VN-Index duy trì xu hướng tăng trong năm 2026.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 00:05:00 +0700</t>
+          <t>Wed, 13 May 26 00:08:00 +0700</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://cafef.vn/tien-lon-chon-loc-chuyen-gia-chi-ten-nhom-co-phieu-xep-hang-cao-tren-thi-truong-188260512213550455.chn</t>
+          <t>https://cafef.vn/them-cong-ty-chung-khoan-ha-du-phong-vn-index-nam-2026-188260512213008592.chn</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VN-Index áp sát đỉnh lịch sử, CTCK cảnh báo kịch bản “xanh vỏ đỏ lòng”</t>
+          <t>Theo dấu dòng tiền cá mập 12/05: Khối ngoại và tự doanh lại cùng bán ròng, FPT tiếp tục thành tâm điểm</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>VNDirect khuyến nghị chiến lược giao dịch linh hoạt, tận dụng cơ hội chốt lời quanh vùng đỉnh và xem xét giải ngân trở lại nếu chỉ số về vùng hỗ trợ quanh 1.820 điểm.</t>
+          <t>Trong phiên thị trường chứng khoán bật tăng trong phiên chiều đầy hứng khởi, khối tự doanh công ty chứng khoán và nhà đầu tư nước ngoài lại đồng thuận bán ròng.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 00:04:00 +0700</t>
+          <t>Tue, 12 May 2026 19:38:00 +0700</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://cafef.vn/vn-index-ap-sat-dinh-lich-su-ctck-canh-bao-kich-ban-xanh-vo-do-long-188260512212732752.chn</t>
+          <t>http://vietstock.vn/2026/05/theo-dau-dong-tien-ca-map-1205-khoi-ngoai-va-tu-doanh-lai-cung-ban-rong-fpt-tiep-tuc-thanh-tam-diem-830-1441753.htm</t>
         </is>
       </c>
     </row>
@@ -1878,25 +1878,25 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Một công ty chứng khoán vốn nghìn tỷ bị phạt nặng</t>
+          <t>Gần 7 triệu cổ phiếu sang tay, STB lập đỉnh</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Chứng khoán Bảo Minh bị xử phạt tổng cộng 780.000.000 đồng do hàng loạt sai phạm.</t>
+          <t>Sau pha điều chỉnh ở phiên trước, thị trường chứng khoán hôm nay (12/5) hồi phục trở lại khi VN-Index lấy lại mốc 1.900 điểm. Dòng tiền tập trung vào nhóm ngân hàng và dầu khí, trong đó STB trở thành tâm điểm với mức tăng cận trần, lập đỉnh giá lịch sử mới.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Wed, 13 May 26 00:02:00 +0700</t>
+          <t>Tue, 12 May 26 18:24:00 +0700</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://cafef.vn/mot-cong-ty-chung-khoan-von-nghin-ty-bi-phat-nang-188260512212628665.chn</t>
+          <t>https://cafef.vn/gan-7-trieu-co-phieu-sang-tay-stb-lap-dinh-188260512174905008.chn</t>
         </is>
       </c>
     </row>
@@ -1908,25 +1908,25 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Quy mô tài sản truyền thống lên tới 1,6 nghìn tỷ USD, Việt Nam có tiềm năng lớn mã hóa tài sản thực</t>
+          <t>VN-Index trở lại mốc 1.900 điểm, dòng tiền tìm đến cổ phiếu bất động sản</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Chuyên gia tài chính cấp cao đến từ Singapore cho rằng khung pháp lý và sự ủng hộ từ Chính phủ sẽ tiếp tục đóng vai trò quan trọng trong quá trình phát triển của thị trường tài sản mã hóa.</t>
+          <t>Thị trường chứng khoán ngày 12-5 ghi nhận nhịp hồi phục đáng chú ý khi VN-Index lấy lại mốc 1.900 điểm sau phiên rung lắc mạnh đầu ngày</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 21:23:00 +0700</t>
+          <t>Tue, 12 May 26 17:52:00 +0700</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://cafef.vn/quy-mo-tai-san-truyen-thong-len-toi-16-nghin-ty-usd-viet-nam-co-tiem-nang-lon-ma-hoa-tai-san-thuc-188260512212342162.chn</t>
+          <t>https://cafef.vn/vn-index-tro-lai-moc-1900-diem-dong-tien-tim-den-co-phieu-bat-dong-san-188260512175253.chn</t>
         </is>
       </c>
     </row>
@@ -1938,437 +1938,437 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kiểm soát hoạt động của người hành nghề môi giới chứng khoán trên mạng xã hội</t>
+          <t>Cổ phiếu Sacombank (STB) tăng cận trần sau biến động nhân sự cấp cao</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Cần rà soát hoạt động của môi giới chứng khoán nhằm bảo đảm không thực hiện những hoạt động khuyến nghị, tư vấn vượt quá phạm vi.</t>
+          <t>Cổ phiếu STB của Sacombank bất ngờ trở thành tâm điểm hút dòng tiền từ các nhà đầu tư trong phiên 12/5, khi tăng cận trần – lập đỉnh giá lịch sử mới ngay sau thông tin ngân hàng bổ nhiệm nhân sự cấp cao.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 17:52:00 +0700</t>
+          <t>Tue, 12 May 26 16:44:00 +0700</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://cafef.vn/kiem-soat-hoat-dong-cua-nguoi-hanh-nghe-moi-gioi-chung-khoan-tren-mang-xa-hoi-188260512175208987.chn</t>
+          <t>https://cafef.vn/co-phieu-sacombank-stb-tang-can-tran-sau-bien-dong-nhan-su-cap-cao-188260512160131532.chn</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Tự doanh CTCK liên tục bán ra hàng trăm tỷ đồng một cổ phiếu họ Gelex</t>
+          <t>Blog chứng khoán: Thanh khoản giảm mạnh, thị trường “xoay trụ”?</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tự doanh CTCK bán ròng 164 tỷ đồng trên HOSE.</t>
+          <t>Ảnh hưởng của c#225;c cổ phiếu vốn h#243;a lớn nhất l#224; VIC, VHM, VCB kh#244;ng qu#225; mạnh trong khi kh#225; nhiều blue-chips tầm trung lại mạnh l#234;n. VNI được neo giữ tốt tạo điều kiện cho số lớn cổ phiếu phục hồi.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 17:48:00 +0700</t>
+          <t>Tue, 12 May 2026 09:16:01 GMT</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://cafef.vn/tu-doanh-ctck-lien-tuc-ban-ra-hang-tram-ty-dong-mot-co-phieu-ho-gelex-188260512174822907.chn</t>
+          <t>https://vneconomy.vn/blog-chung-khoan-thanh-khoan-giam-manh-thi-truong-xoay-tru.htm</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Đại diện UBCKNN: Khi nào có sàn giao dịch tài sản mã hoá đầu tiên phụ thuộc hoàn toàn vào năng lực của doanh nghiệp</t>
+          <t>VN-Index quay lại mốc 1.900 điểm</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Liên quan tới lộ trình triển khai thị trường tài sản mã hóa chính thức, ông Hòa cho biết tiến độ hiện nay không phụ thuộc vào cơ quan quản lý mà phụ thuộc chủ yếu vào năng lực của doanh nghiệp.</t>
+          <t>Bất chấp hai cổ phiếu "họ" Vingroup tiếp tục giảm, VN-Index vẫn tăng hơn 5 điểm, lên 1.901 điểm nhờ trạng thái hưng phấn của nhóm dầu khí và một số mã ngân hàng.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 16:53:00 +0700</t>
+          <t>Tue, 12 May 2026 16:10:36 +0700</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://cafef.vn/dai-dien-ubcknn-bao-gio-co-san-giao-dich-tai-san-ma-hoa-dau-tien-phu-thuoc-hoan-toan-vao-nang-luc-cua-doanh-nghiep-188260512165347989.chn</t>
+          <t>https://vnexpress.net/vn-index-quay-lai-moc-1-900-diem-5073096.html</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Doanh nghiệp Trung Quốc thâu tóm 'ông lớn' thuốc kháng sinh Imexpharm</t>
+          <t>Ước tính 17/26 ngân hàng niêm yết không đạt tỷ lệ cấp tín dụng so với huy động vốn theo tiêu chí mới</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Lian SGP Holding thuộc tập đoàn Livzon Pharmaceutical (Trung Quốc) vừa mua 68% vốn và trở thành cổ đông lớn nhất của doanh nghiệp đứng đầu mảng thuốc kháng sinh Imexpharm.</t>
+          <t>Chứng kho#225;n Rồng Việt (VDSC) ước t#237;nh c#243; 17/26 ng#226;n h#224;ng ni#234;m yết kh#244;ng đạt tỷ lệ cấp t#237;n dụng so với huy động vốn (CDR) trong qu#253; 1/2026 nếu chiếu theo quy định mới dự kiến, như một c#225;ch để h#236;nh dung th#225;ch thức rất lớn trong hai năm tới li#234;n quan chi ph#237; tu#226;n thủ.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 16:21:11 +0700</t>
+          <t>Tue, 12 May 2026 06:52:14 GMT</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/doanh-nghiep-trung-quoc-thau-tom-ong-lon-thuoc-khang-sinh-imexpharm-5073089.html</t>
+          <t>https://vneconomy.vn/uoc-tinh-1726-ngan-hang-niem-yet-khong-dat-ty-le-cap-tin-dung-so-voi-huy-dong-von-theo-tieu-chi-moi.htm</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Trao quyền chọn tài sản mã hóa niêm yết cho các sàn giao dịch</t>
+          <t>SJC lãi kỷ lục dù doanh thu thấp nhất 10 năm</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Về phía quyền lợi và nghĩa vụ chuyên môn, các tổ chức sẽ có một quyền rất quan trọng là quyền lựa chọn tài sản mã hóa để niêm yết và giao dịch theo thông lệ quốc tế, song lãnh đạo UBCKNN khuyến khích sự thận trọng, ưu tiên các tài sản có tính thanh khoản cao và phổ biến để hạn chế rủi ro cho thị trường.</t>
+          <t>Doanh thu ở mức thấp nhất một thập kỷ, Công ty SJC vẫn có lợi nhuận sau thuế tăng 9% lên mức kỷ lục 425,5 tỷ đồng năm ngoái.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 15:53:00 +0700</t>
+          <t>Tue, 12 May 2026 12:13:58 +0700</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://cafef.vn/trao-quyen-chon-tai-san-ma-hoa-niem-yet-cho-cac-san-giao-dich-188260512155331827.chn</t>
+          <t>https://vnexpress.net/sjc-lai-ky-luc-du-doanh-thu-thap-nhat-10-nam-5072912.html</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Gần 800 triệu cổ phiếu Hoà Phát sắp về tài khoản nhà đầu tư</t>
+          <t>Loại trừ nhóm Vingroup, định giá thị trường ngày càng rẻ hơn</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sau đợt chia này, lượng cổ phiếu lưu hành của Hoà Phát sẽ tăng lên hơn 8,4 tỷ cổ phiếu - tương đương dân số toàn cầu.</t>
+          <t>Khi d#242;ng tiền đầu cơ theo đuổi lợi nhuận ngắn hạn v#224; v#224;o một nh#243;m cổ phiếu định gi#225; rất cao, thị trường lại bắt đầu cho ch#250;ng ta những cơ hội đầu tư c#225;c doanh nghiệp c#243; kết quả kinh doanh t#237;ch cực với định gi#225; rẻ nhưng bị d#242;ng tiền bỏ qua.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 15:32:00 +0700</t>
+          <t>Mon, 11 May 2026 12:49:46 GMT</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://cafef.vn/gan-800-trieu-co-phieu-hoa-phat-sap-ve-tai-khoan-nha-dau-tu-188260512153307166.chn</t>
+          <t>https://vneconomy.vn/loai-tru-nhom-vingroup-dinh-gia-thi-truong-ngay-cang-re-hon.htm</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Lừa đảo trực tuyến hơn 8.000 tỷ đồng năm 2025: Chuyên gia chỉ ra ‘bí kíp’ thúc đẩy niểm tin tài chính số trong kỷ nguyên AI</t>
+          <t>Blue-chips giảm la liệt, “tiền nóng” co cụm</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Đại tá Nguyễn Hồng Quân, Phó Cục trưởng Cục An ninh mạng và phòng, chống tội phạm sử dụng công nghệ cao, Phó Chủ tịch Liên minh Niềm tin số, nêu bật "nhiệm vụ" chung để nâng cao niềm tin số tài chính trong kỷ nguyên AI.</t>
+          <t>Gần như to#224;n bộ cổ phiếu trong rổ blue-chips VN30 lao dốc chiều nay, bao gồm cả c#225;c trụ dẫn VIC, VHM. Điều ng#224;y ngay lập tức t#225;c động đến VN-Index, đẩy chỉ số n#224;y đảo chiều giảm 1,04% v#224; đ#225;nh mất lu#244;n mốc 1900 điểm.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 15:18:00 +0700</t>
+          <t>Mon, 11 May 2026 08:27:18 GMT</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://cafef.vn/lua-dao-truc-tuyen-hon-8000-ty-dong-nam-2025-chuyen-gia-chi-ra-bi-kip-thuc-day-niem-tin-tai-chinh-so-trong-ky-nguyen-ai-188260512151809266.chn</t>
+          <t>https://vneconomy.vn/blue-chips-giam-la-liet-tien-nong-co-cum.htm</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cổ đông liên quan Thành viên HĐQT Vinasun muốn thoái sạch vốn</t>
+          <t>MSR đạt doanh thu gần 3.000 tỷ trong quý I</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Tư vấn Kim Ngưu vừa đăng ký bán ra toàn bộ hơn 3,4 triệu cổ phiếu VNS nhằm mục đích cơ cấu danh mục đầu tư. Nếu giao dịch thành công, doanh nghiệp này sẽ rời ghế cổ đông tại Vinasun.</t>
+          <t>Doanh thu Masan High-Tech Materials (MSR) tăng gần 115% so với cùng kỳ, đạt 2.993 tỷ trong quý I/2026 nhờ sự cải thiện đồng thời của giá hàng hóa, sản lượng và cấu trúc tài chính.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 14:39:00 +0700</t>
+          <t>Mon, 11 May 2026 09:00:00 +0700</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://cafef.vn/co-dong-lien-quan-thanh-vien-hdqt-vinasun-muon-thoai-sach-von-188260512143443164.chn</t>
+          <t>https://vnexpress.net/msr-dat-doanh-thu-gan-3-000-ty-trong-quy-i-5072256.html</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VnExpress Business</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Thứ trưởng Bộ Tài chính: Sớm nhất trong quý 3 có thể vận hành thị trường tài sản mã hóa</t>
+          <t>Chuỗi nhà thuốc của Thế Giới Di Động sắp hết lỗ</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Thứ trưởng Bộ Tài chính Nguyễn Đức Chi chia sẻ những thông tin quan trọng về tiến trình xây dựng thị trường tài sản mã hóa tại Việt Nam</t>
+          <t>Thế Giới Di Động cho biết chuỗi nhà thuốc An Khang "gần ngưỡng hòa vốn" và có thể đóng góp lợi nhuận sau khoảng 8 năm doanh nghiệp này tham gia mảng bán lẻ dược.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 14:38:00 +0700</t>
+          <t>Mon, 11 May 2026 00:02:00 +0700</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://cafef.vn/thu-truong-bo-tai-chinh-som-nhat-trong-quy-3-co-the-van-hanh-thi-truong-tai-san-ma-hoa-188260512143753521.chn</t>
+          <t>https://vnexpress.net/chuoi-nha-thuoc-cua-the-gioi-di-dong-sap-het-lo-5072234.html</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Doanh nghiệp dược hàng đầu Việt Nam chính thức về tay “gã khổng lồ” Trung Quốc</t>
+          <t>Sau tái cấu trúc, Nam Hoa (NHT) hoạt động có lãi, trả cổ tức bằng tiền mặt 30%</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Giá trị giao dịch ước tính vào khoảng 6.000 tỷ đồng.</t>
+          <t>Hội đồng quản trị C#244;ng ty Cổ phần Sản xuất v#224; Thương mại Nam Hoa (m#227; chứng kho#225;n: NHT) vừa th#244;ng qua nghị quyết chi trả cổ tức bằng tiền mặt tỷ lệ 30% cho năm 2025 (tương ứng 3.000 đồng/cổ phiếu). Đ#226;y l#224; mức chi trả cao, phản #225;nh sự phục hồi ấn tượng v#224; d#242;ng tiền ổn định của doanh nghiệp sau giai đoạn t#225;i cấu tr#250;c mạnh mẽ…</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 13:46:00 +0700</t>
+          <t>Sun, 10 May 2026 03:40:28 GMT</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://cafef.vn/doanh-nghiep-duoc-hang-dau-viet-nam-chinh-thuc-ve-tay-ga-khong-lo-trung-quoc-188260512134636898.chn</t>
+          <t>https://vneconomy.vn/sau-tai-cau-truc-nam-hoa-nht-hoat-dong-co-lai-tra-co-tuc-bang-tien-mat-30.htm</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EU rót hơn 230 tỷ USD vào pin, xe điện để giảm phụ thuộc Trung Quốc</t>
+          <t>Nhà đầu tư cá nhân mua ròng 1.200 tỷ phiên cuối tuần, tiếp tục mạnh tay gom FPT</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Châu Âu và Thụy Sĩ đầu tư 235 tỷ USD vào chuỗi cung ứng pin, xe điện và trạm sạc, nhằm định hình hệ sinh thái và giảm phụ thuộc vào Trung Quốc.</t>
+          <t>Nh#224; đầu tư c#225; nh#226;n tuần qua mua r#242;ng 1221,4 tỷ đồng, trong đ#243; họ mua r#242;ng khớp lệnh l#224; 809,9 tỷ đồng.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Tue, 12 May 2026 12:05:00 +0700</t>
+          <t>Sun, 10 May 2026 03:02:35 GMT</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/eu-rot-hon-230-ty-usd-vao-pin-xe-dien-de-giam-phu-thuoc-trung-quoc-5072856.html</t>
+          <t>https://vneconomy.vn/nha-dau-tu-ca-nhan-mua-rong-1200-ty-phien-cuoi-tuan-tiep-tuc-manh-tay-gom-fpt.htm</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Gemadept chốt ngày chi hơn 938 tỷ đồng trả cổ tức năm 2025</t>
+          <t>Cuộc đua tăng vốn: Các công ty chứng khoán tăng thêm 100.000 tỷ trong năm 2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Ngày 22/5/2026 tới đây, Gemadept sẽ chốt danh sách cổ đông để thực hiện chi trả cổ tức năm 2025 bằng tiền mặt với tỷ lệ 22%. Ngày thanh toán dự kiến 29/5/2026.</t>
+          <t>Tổng quy m#244; tăng vốn to#224;n ng#224;nh năm 2026 ước t#237;nh c#243; thể tiếp tục duy tr#236; ở mức cao tương đương 2025 (~100 ngh#236;n tỷ đồng).</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 10:51:00 +0700</t>
+          <t>Sat, 09 May 2026 12:40:53 GMT</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>https://cafef.vn/gemadept-chot-ngay-chi-hon-938-ty-dong-tra-co-tuc-nam-2025-188260512094843159.chn</t>
+          <t>https://vneconomy.vn/cuoc-dua-tang-von-cac-cong-ty-chung-khoan-tang-them-100000-ty-trong-nam-2026.htm</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Sẽ đưa Blockchain, Big data, AI vào hoạt động giám sát thị trường; sớm nhất trong quý 3 sẽ vận hành thị trường tài sản mã hoá chính thức tại Việt Nam</t>
+          <t>Thị trường chứng khoán Việt Nam  2025 và triển vọng 2026</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Đại diện UBCKNN cho biết thời gian tới sẽ đưa công nghệ chuỗi khối (blockchain), dữ liệu lớn (big data) và trí tuệ nhân tạo (AI) vào hoạt động giám sát thị trường thông qua hệ thống thông tin tổng thể và kho dữ liệu tập trung.</t>
+          <t>Thị trường chứng kho#225;n (TTCK) Việt Nam trong năm 2025 trải qua nhiều phi#234;n tăng giảm đan xen nhưng nh#236;n chung duy tr#236; hoạt động ổn định v#224; ghi nhận những kết quả nổi bật nhờ sự hỗ trợ t#237;ch cực từ nền tảng kinh tế vĩ m#244; trong nước v#224; sự chỉ đạo, điều h#224;nh chủ động, linh hoạt, quyết liệt của Ch#237;nh phủ, Thủ tướng Ch#237;nh phủ.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 10:44:00 +0700</t>
+          <t>Sat, 09 May 2026 02:00:00 GMT</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://cafef.vn/se-dua-blockchain-big-data-ai-vao-hoat-dong-giam-sat-thi-truong-som-nhat-trong-quy-3-se-van-hanh-thi-truong-tai-san-ma-hoa-chinh-thuc-tai-viet-nam-188260512104430607.chn</t>
+          <t>https://vneconomy.vn/thi-truong-chung-khoan-viet-nam-2025-va-trien-vong-2026.htm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CafeF</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Lãnh đạo doanh nghiệp hé lộ lý do đề xuất xây 2 toà tháp tưởng niệm giữa trung tâm Hà Nội</t>
+          <t>“Lệch pha” ngày càng rõ, VN-Index áp sát ngưỡng 1920 điểm, cổ phiếu đỏ la liệt</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Lý giải việc điều chỉnh quy hoạch, ông Đinh Ngọc Dương cho rằng mô hình “công viên nhà tang lễ” là hướng tiếp cận mới nhằm đáp ứng nhu cầu tổ chức tang lễ văn minh hơn tại đô thị lớn, với nhiều không gian xanh và trải nghiệm tiễn biệt mang tính nhân văn hơn.</t>
+          <t>VN-Index nh#237;ch th#234;m 6,36 điểm trong phi#234;n h#244;m nay tiến l#234;n mức 1915,37 điểm. Chỉ “nhấn” th#234;m ch#250;t nữa l#224; chỉ số c#243; đỉnh cao lịch sử mới v#224; điều n#224;y ho#224;n to#224;n khả thi nếu VIC, VHM tiếp tục mạnh. Tuy nhi#234;n nh#224; đầu tư c#243; hưởng lợi hay kh#244;ng lại l#224; vấn đề kh#225;c.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Tue, 12 May 26 10:10:00 +0700</t>
+          <t>Fri, 08 May 2026 08:49:38 GMT</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://cafef.vn/lanh-dao-doanh-nghiep-he-lo-ly-do-de-xuat-xay-2-toa-thap-tuong-niem-giua-trung-tam-ha-noi-188260512100853346.chn</t>
+          <t>https://vneconomy.vn/lech-pha-ngay-cang-ro-vn-index-ap-sat-nguong-1920-diem-co-phieu-do-la-liet.htm</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>'Cá voi' Bitcoin trị giá 40 triệu USD thức giấc</t>
+          <t>Hơn nửa số mã dầu khí vẫn giữ xu hướng tăng dài hạn suốt 5 tháng</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Sau hơn 10 năm nắm giữ, một nhà đầu tư đã chuyển lượng Bitcoin trị giá 40 triệu USD sang ví mới trong bối cảnh tiền số phục hồi.</t>
+          <t>Sau nhịp tăng mạnh đầu năm 2026, nhóm dầu khí đã trải qua giai đoạn điều chỉnh sâu khi hàng loạt cổ phiếu đầu ngành giảm 30-50% so với vùng đỉnh gần nhất. Tuy nhiên, dòng tiền tại nhóm này vẫn chưa rút lui hoàn toàn khi hơn 50% số mã được theo dõi đã duy trì xu hướng tăng dài hạn trong 5 tháng.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 21:19:05 +0700</t>
+          <t>Thu, 14 May 2026 09:02:00 +0700</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -2376,29 +2376,29 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/ca-voi-bitcoin-tri-gia-40-trieu-usd-thuc-giac-5072749.html</t>
+          <t>http://vietstock.vn/2026/05/hon-nua-so-ma-dau-khi-van-giu-xu-huong-tang-dai-han-suot-5-thang-830-1442029.htm</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VN-Index giảm gần 20 điểm phiên đầu tuần</t>
+          <t>Quỹ Đầu tư do bà Nguyễn Thanh Phượng làm Chủ tịch bán hết cổ phiếu VCI</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Bốn cổ phiếu liên quan đến Vingroup đều giảm, dao động 1-6,5%, trở thành tác nhân chính khiến VN-Index mất gần 20 điểm trong phiên đầu tuần.</t>
+          <t>Quỹ Đầu tư Bản Việt Discovery bán ra toàn bộ 135.000 cổ phiếu VCI trong thời gian từ 6-8/5/2026, qua đó không còn là cổ đông của Vietcap.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 15:49:54 +0700</t>
+          <t>Thu, 14 May 26 08:30:00 +0700</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2406,29 +2406,29 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/vn-index-giam-gan-20-diem-phien-dau-tuan-5072618.html</t>
+          <t>https://cafef.vn/quy-dau-tu-do-ba-nguyen-thanh-phuong-lam-chu-tich-ban-het-co-phieu-vci-188260514080941252.chn</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VN-Index được dự đoán sớm vượt 2.000 điểm</t>
+          <t>Top cổ phiếu đáng chú ý đầu phiên 14/05</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Nhiều nhóm phân tích cho rằng VN-Index tháng này có thể vượt 2.000 điểm nhờ lực kéo từ cổ phiếu trụ và thanh khoản dồi dào.</t>
+          <t>Danh sách các mã cổ phiếu tăng và giảm mạnh nhất những phiên gần đây theo số liệu thống kê của Vietstock.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Mon, 11 May 2026 00:05:00 +0700</t>
+          <t>Thu, 14 May 2026 08:00:00 +0700</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2436,29 +2436,29 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/vn-index-duoc-du-doan-som-vuot-2-000-diem-5072145.html</t>
+          <t>http://vietstock.vn/2026/05/top-co-phieu-dang-chu-y-dau-phien-1405-830-1442191.htm</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>Vietstock</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Sổ đỏ cấp sai quy định được xem xét điều chỉnh, nộp bổ sung thuế</t>
+          <t>14/05: Đọc gì trước giờ giao dịch chứng khoán?</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Các dự án được cấp sổ đỏ sai quy định trước đây sẽ được xem xét điều chỉnh và nộp bổ sung nghĩa vụ tài chính, theo cơ chế đặc thù của Chính phủ.</t>
+          <t>Cùng điểm lại những tin tức tài chính - kinh tế trong nước và quốc tế đáng chú ý trong 24h qua trước giờ giao dịch hôm nay.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Sun, 10 May 2026 17:40:04 +0700</t>
+          <t>Thu, 14 May 2026 06:02:00 +0700</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/so-do-cap-sai-quy-dinh-duoc-xem-xet-dieu-chinh-nop-bo-sung-thue-5072135.html</t>
+          <t>http://vietstock.vn/2026/05/1405-doc-gi-truoc-gio-giao-dich-chung-khoan-830-1442326.htm</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Đề xuất doanh nghiệp nộp thuế thay người gom ve chai, phế liệu</t>
+          <t>Hà Nội có thể cho thuê vỉa hè 45.000 đồng một m2 mỗi tháng để kinh doanh</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>VCCI đề nghị Bộ Tài chính bổ sung cơ chế khai, nộp thuế thay với hộ kinh doanh ve chai, đồng nát và sửa cách tính thuế với mô hình tài xế công nghệ.</t>
+          <t>Hà Nội có thể thí điểm cho thuê một phần lòng đường, vỉa hè cao nhất 45.000 đồng một m2 mỗi tháng để phát triển kinh tế đô thị, kinh tế đêm.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Sun, 10 May 2026 12:48:02 +0700</t>
+          <t>Thu, 14 May 2026 05:00:00 +0700</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -2496,29 +2496,29 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/de-xuat-doanh-nghiep-nop-thue-thay-nguoi-gom-ve-chai-phe-lieu-5072084.html</t>
+          <t>https://vnexpress.net/ha-noi-co-the-cho-thue-via-he-45-000-dong-mot-m2-moi-thang-de-kinh-doanh-5073615.html</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>CafeF</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Kinh tế Việt - Ấn: Rộng cửa đón tỷ USD</t>
+          <t>Cổ phiếu từng gây sốt với 20 phiên kịch trần liên tiếp lại "nổi sóng"</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Chuyến thăm Ấn Độ của Tổng Bí thư, Chủ tịch nước Tô Lâm mở ra dư địa thúc đẩy thương mại song phương, hướng tới mục tiêu 25 tỷ USD vào năm 2030.</t>
+          <t>Thị giá nhờ đó tăng một mạch từ vùng 30.000 đồng lên sát 100.000 đồng, tương ứng tăng xấp xỉ 220% chỉ sau khoảng 1 tháng.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Sun, 10 May 2026 07:00:07 +0700</t>
+          <t>Thu, 14 May 26 00:06:00 +0700</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/kinh-te-viet-an-rong-cua-don-ty-usd-5072031.html</t>
+          <t>https://cafef.vn/co-phieu-tung-gay-sot-voi-20-phien-kich-tran-lien-tiep-lai-noi-song-188260513223933796.chn</t>
         </is>
       </c>
     </row>
@@ -2538,17 +2538,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Việt Nam chi gần tỷ USD nhập hạt điều trong một tháng</t>
+          <t>Cú hích tái cấu trúc kinh tế toàn cầu từ xung đột Trung Đông</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Là nước xuất khẩu điều nhân lớn nhất thế giới, nhưng riêng tháng 4, các doanh nghiệp Việt đã chi gần 943 triệu USD để nhập khẩu điều thô.</t>
+          <t>Dù gây thiệt hại ngắn hạn, xung đột Trung Đông được giới phân tích xem là cú hích buộc thế giới định hình lại chuỗi cung ứng năng lượng dài hạn.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Sat, 09 May 2026 19:58:16 +0700</t>
+          <t>Thu, 14 May 2026 00:05:00 +0700</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -2556,29 +2556,29 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/viet-nam-chi-gan-ty-usd-nhap-hat-dieu-trong-mot-thang-5071916.html</t>
+          <t>https://vnexpress.net/cu-hich-tai-cau-truc-kinh-te-toan-cau-tu-xung-dot-trung-dong-5073241.html</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>VnExpress Business</t>
+          <t>VNeconomy</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Có nên bán nhà Hà Nội khi giá đã giảm 1 tỷ đồng?</t>
+          <t>Thị trường vẫn đang tìm điểm cân bằng mới và giao dịch khá lỏng lẻo</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Theo chuyên gia, thị trường bất động sản không trả tiền theo "ký ức" mà theo khả năng, cần đưa ra giá bán phù hợp với thanh khoản thực tế.</t>
+          <t>VnEconomy giới thiệu nhận định v#224; khuyến nghị đầu tư của một số c#244;ng ty chứng kho#225;n về diễn biến thị trường ng#224;y 14/5/2026</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Sat, 09 May 2026 13:00:55 +0700</t>
+          <t>Wed, 13 May 2026 14:24:07 GMT</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -2586,37 +2586,2137 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>https://vnexpress.net/co-nen-ban-nha-ha-noi-khi-gia-da-giam-1-ty-dong-5071849.html</t>
+          <t>https://vneconomy.vn/thi-truong-van-dang-tim-diem-can-bang-moi-va-giao-dich-kha-long-leo.htm</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Tự doanh CTCK bán ròng gần 400 tỷ trong phiên 13/5, cổ phiếu nào là tâm điểm?</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Tự doanh CTCK bán ròng 379 tỷ đồng trên HOSE.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 18:44:00 +0700</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/tu-doanh-ctck-ban-rong-gan-400-ty-trong-phien-13-5-co-phieu-nao-la-tam-diem-188260513184457858.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>VnExpress Business</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Công ty điện mặt trời của Trung Nam lỗ gần 1.000 tỷ đồng</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Trung Nam Thuận Nam, chủ đầu tư nhà máy điện mặt trời 450 MW ở Khánh Hòa, năm ngoái lỗ trước thuế 970 tỷ đồng, nâng lỗ lũy kế lên trên 1.800 tỷ.</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Fri, 08 May 2026 12:32:52 +0700</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>https://vnexpress.net/cong-ty-dien-mat-troi-cua-trung-nam-lo-gan-1-000-ty-dong-5071456.html</t>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Gia Lai đề xuất xây trung tâm đấu giá cá ngừ đầu tiên Đông Nam Á</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>UBND tỉnh Gia Lai đề xuất đầu tư cảng cá thông minh Tam Quan, hướng tới hình thành trung tâm logistics thủy sản và trung tâm đấu giá cá ngừ đại dương đầu tiên ở Đông Nam Á.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 18:30:33 +0700</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/gia-lai-de-xuat-xay-trung-tam-dau-gia-ca-ngu-dau-tien-dong-nam-a-5073426.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Vietstock Daily 14/05/2026: Phân hóa rõ nét</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>VN-Index rung lắc mạnh khi test lại đỉnh cũ tháng 01/2026 (tương đương vùng 1,900-1,920 điểm). Chỉ báo Stochastic Oscillator tiếp tục giảm trong khi MACD cũng đang thu hẹp khoảng cách với đường signal. Nếu chỉ báo này cắt xuống đường signal trong các phiên tới thì rủi ro ngắn hạn sẽ gia tăng.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 18:10:03 +0700</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/vietstock-daily-14052026-phan-hoa-ro-net-1636-1442207.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Cổ đông lớn sang tay cổ phiếu CK8 giữa nguy cơ hủy tư cách đại chúng</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Bà Ngô Thị Minh Phương trở thành cổ đông lớn của CTCP Cơ khí 120 (UPCoM: CK8) sau khi mua vào 665.8 ngàn cổ phiếu. Ở chiều ngược lại, bà Trần Thị Yến Hà đã bán ra đúng bằng số lượng này và thoái sạch vốn CK8. Thương vụ sang tay diễn ra trong bối cảnh công ty đang đối mặt với nguy cơ bị hủy tư cách đại chúng do vốn chủ sở hữu rớt xuống mức âm.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 17:20:45 +0700</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/co-dong-lon-sang-tay-co-phieu-ck8-giua-nguy-co-huy-tu-cach-dai-chung-739-1442149.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>"Vàng đang trên đà vọt lên 10.000 USD", một tỷ phú dồn cả tỷ USD mua vàng, bạc dù vừa "thua đau đớn"</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Có một người đàn ông đang đặt cược 98% gia tài tỷ USD của mình vào kim loại quý, ngay giữa lúc thị trường rung lắc dữ dội nhất.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 16:48:00 +0700</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/vang-dang-tren-da-vot-len-10000-usd-mot-ty-phu-don-ca-ty-usd-mua-vang-bac-du-vua-thua-dau-don-188260513164354302.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Nhịp đập Thị trường 13/05: Khối ngoại liên tục bán ròng, VN-Index cheo leo tại mốc 1,900 điểm</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Kết thúc phiên giao dịch, VN-Index giảm 2.73 điểm (-0.14%), xuống mức 1,898.37 điểm; HNX-Index tăng 1.34 điểm (+0.53%), lên mức 254.62 điểm. Độ rộng toàn thị trường với sắc đỏ lấn lướt khi bên bán có 353 mã giảm và bên mua có 335 mã tăng. Tương tự, sắc đỏ lấn lướt trong rổ VN30 với 15 mã giảm, 13 mã tăng và 2 mã tham chiếu.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 16:47:00 +0700</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/nhip-dap-thi-truong-1305-khoi-ngoai-lien-tuc-ban-rong-vn-index-cheo-leo-tai-moc-1900-diem-1636-1441856.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Đơn vị vận hành HoSE và HNX lên kế hoạch lãi kỷ lục</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Sở Giao dịch chứng khoán Việt Nam dự kiến có lãi kỷ lục 2.987 tỷ đồng năm nay với nhiều kế hoạch như ETF vàng, sàn carbon và startup.</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 16:35:03 +0700</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/don-vi-van-hanh-hose-va-hnx-len-ke-hoach-lai-ky-luc-5073472.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Một doanh nghiệp đầu ngành sắp lăn chốt cổ tức tiền mặt 83%, "đại gia" Thái Lan vớ bẫm</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Đây cũng là mức cổ tức tiền mặt cao nhất trong lịch sử hoạt động của doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 16:11:00 +0700</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/mot-doanh-nghiep-dau-nganh-sap-lan-chot-co-tuc-tien-mat-83-dai-gia-thai-lan-vo-bam-188260513161023867.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>​Chuyên gia quốc tế: Việt Nam có cơ hội thành 'tọa độ vàng' siêu sự kiện</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Chính sách mở đường và làn sóng đầu tư hạ tầng quy mô lớn đang tạo đà cho nền công nghiệp văn hóa Việt Nam bứt phá, vươn tầm thành điểm đến mới của kinh tế trải nghiệm toàn cầu.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 16:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/chuyen-gia-quoc-te-viet-nam-co-co-hoi-thanh-toa-do-vang-sieu-su-kien-5073499.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Fecon sắp phát hành lô trái phiếu 125 tỷ đồng</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Fecon dự kiến phát hành 1.250 trái phiếu mã FCN12601 ra thị trường trong nước vào ngày 15/5/2026, mệnh giá 100 triệu đồng/trái phiếu, qua đó huy động 125 tỷ đồng.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 15:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/fecon-sap-phat-hanh-lo-trai-phieu-125-ty-dong-188260513144942479.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Ngân hàng tiếp tục rao bán nhà máy nông sản hơn 1.200 tỷ liên quan bà Trương Mỹ Lan</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>VietinBank phát mãi lần hai nhà máy Tanifood Tây Ninh liên quan vụ án Vạn Thịnh Phát với giá khởi điểm 1.200 tỷ đồng, thấp hơn 10% so với lần rao bán trước.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 15:47:20 +0700</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/ngan-hang-tiep-tuc-rao-ban-nha-may-nong-san-hon-1-200-ty-lien-quan-ba-truong-my-lan-5073438.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Phiên 13/5: Khối ngoại tiếp đà bán ròng nghìn tỷ, ngược chiều gom mạnh một cổ phiếu ngân hàng</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Giao dịch của khối ngoại là điểm trừ khi bán ròng khoảng 1.475 tỷ đồng.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 15:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/phien-13-5-khoi-ngoai-tiep-da-ban-rong-nghin-ty-nguoc-chieu-gom-manh-mot-co-phieu-ngan-hang-1882605131542172.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Dòng tiền mạnh lên, thị trường phân hóa</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Thanh khoản khớp lệnh hai s#224;n chiều nay tăng 67% so với buổi s#225;ng, trong đ#243; HoSE tăng gần 69% l#234;n mức cao nhất 7 tuần. Độ rộng cho thấy cổ phiếu c#243; sự phục hồi kh#225; tốt, mặc d#249; ảnh hưởng của trụ khiến VN-Index kh#244;ng thể vượt qua tham chiếu.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 08:33:54 GMT</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/dong-tien-manh-len-thi-truong-phan-hoa.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Vừa về tay ông lớn dược phẩm Trung Quốc, loạt lãnh đạo Imexpharm cùng bán ra lượng cổ phiếu</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Nhiều lãnh đạo của Công ty cổ phần Dược phẩm Imexpharm (MCK: IMP, sàn: HoSE) vừa báo cáo kết quả bán ra cổ phiếu.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 15:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/vua-ve-tay-ong-lon-duoc-pham-trung-quoc-loat-lanh-dao-imexpharm-cung-ban-ra-luong-co-phieu-188260513145031724.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Người nhà lãnh đạo SeABank đăng ký mua 5 triệu cổ phiếu SSB</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Ông Lê Hữu Báu, chồng của bà Nguyễn Thị Nga- Phó Chủ tịch thường trực HĐQT SeABank, vừa đăng ký mua 5 triệu cổ phiếu SSB nhằm mục đích tăng tỷ lệ sở hữu.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 15:18:00 +0700</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/nguoi-nha-lanh-dao-seabank-dang-ky-mua-5-trieu-co-phieu-ssb-188260513145128351.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Một doanh nghiệp “lạ” trả cổ tức kỷ lục 60% bằng tiền mặt</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Đây là công ty duy nhất trên sàn bán các loại kềm.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 14:41:00 +0700</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/mot-doanh-nghiep-la-tra-co-tuc-ky-luc-60-bang-tien-mat-18826051314410115.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Phát hiện giá Bitcoin tương quan với thị trường cá cược thể thao</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Diễn biến giá của Bitcoin và quỹ ETF lớn nhất thế giới về cá cược thể thao có mối liên hệ về mặt thống kê tới hơn 80%.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 14:35:54 +0700</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/phat-hien-gia-bitcoin-tuong-quan-voi-thi-truong-ca-cuoc-the-thao-5073356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Agribank thúc đẩy giải pháp ngân hàng số khu vực Tây Nam Bộ</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Agribank đẩy mạnh các giải pháp thanh toán không tiền mặt, mở rộng hạ tầng giao dịch, thúc đẩy tài chính số khu vực nông thôn Tây Nam Bộ.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 14:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/agribank-thuc-day-giai-phap-ngan-hang-so-khu-vuc-tay-nam-bo-5073401.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Phân tích kỹ thuật phiên chiều 13/05: Tín hiệu trái chiều xuất hiện</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>VN-Index giảm điểm khi tiếp tục kiểm tra lại đỉnh cũ tháng 01/2026 (tương đương vùng 1,900-1,920 điểm). HNX-Index có phiên tăng điểm thứ 3 liên tiếp và  đang nằm trên đường Middle của Bollinger Bands.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 13:03:11 +0700</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/phan-tich-ky-thuat-phien-chieu-1305-tin-hieu-trai-chieu-xuat-hien-585-1442015.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Anpha Petrol nói gì sau khi cổ phiếu tăng trần 5 phiên liền?</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Giai đoạn 04-08/05, cổ phiếu CTCP Tập đoàn Dầu khí An Pha (HOSE: ASP) tăng trần liên tiếp dẫn đến phải giải trình với Sở Giao dịch Chứng khoán TPHCM (HOSE). Ngay trong ngày 08/05, Doanh nghiệp đã đưa ra văn bản chính thức.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 10:49:47 +0700</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/anpha-petrol-noi-gi-sau-khi-co-phieu-tang-tran-5-phien-lien-830-1441846.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>VinFast sẽ tách mảng sản xuất tại Việt Nam</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>VinFast dự kiến chuyển giao mảng sản xuất cho nhóm nhà đầu tư mới với giá khoảng 530 triệu USD và ông Phạm Nhật Vượng vẫn tham gia pháp nhân mới nhưng giảm tỷ lệ sở hữu.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 10:46:42 +0700</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/vinfast-se-tach-mang-san-xuat-tai-viet-nam-5073349.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>FID nhận ‘combo’ cảnh báo, kiểm soát</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Sở Giao dịch Chứng khoán Hà Nội (HNX) vừa ban hành các quyết định liên quan đến việc xử lý vi phạm đối với CTCP Đầu tư và Phát triển Doanh nghiệp Việt Nam (HNX: FID).</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 09:41:32 +0700</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/fid-nhan-8216combo8217-canh-bao-kiem-soat-830-1441642.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Mở tài khoản chứng khoán qua VNeID: Tiện ích hiện đại cho nhà đầu tư</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Hiện nay, b#234;n cạnh c#225;c giao dịch h#224;nh ch#237;nh v#224; ng#226;n h#224;ng, người d#226;n đ#227; c#243; thể thực hiện mở t#224;i khoản chứng kho#225;n trực tiếp th#244;ng qua ứng dụng VNeID của Bộ C#244;ng an. Đ#226;y l#224; bước tiến mới trong việc tận dụng dữ liệu d#226;n cư quốc gia để đơn giản h#243;a thủ tục t#224;i ch#237;nh cho c#244;ng d#226;n.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 02:40:31 GMT</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/mo-tai-khoan-chung-khoan-qua-vneid-tien-ich-hien-dai-cho-nha-dau-tu.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Bà Huỳnh Bích Ngọc muốn bán 15 triệu cổ phiếu AgriS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Bà Huỳnh Bích Ngọc đăng ký bán ra 15 triệu cổ phiếu SBT của AgriS nhằm mục đích cơ cấu danh mục đầu tư.</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 09:34:00 +0700</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/ba-huynh-bich-ngoc-muon-ban-15-trieu-co-phieu-agris-188260513092914186.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Top cổ phiếu đáng chú ý đầu phiên 13/05</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Danh sách các mã cổ phiếu tăng và giảm mạnh nhất những phiên gần đây theo số liệu thống kê của Vietstock.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 08:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/top-co-phieu-dang-chu-y-dau-phien-1305-830-1441641.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13/05: Đọc gì trước giờ giao dịch chứng khoán?</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Cùng điểm lại những tin tức tài chính - kinh tế trong nước và quốc tế đáng chú ý trong 24h qua trước giờ giao dịch hôm nay.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/1305-doc-gi-truoc-gio-giao-dich-chung-khoan-830-1441766.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Giới đầu tư kỳ vọng gì vào thượng đỉnh Mỹ - Trung?</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Giới đầu tư dự báo khó có thỏa thuận kinh tế đột phá, dồn chú ý vào diễn biến lĩnh vực AI tại cuộc gặp lãnh đạo Mỹ - Trung.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 2026 00:08:00 +0700</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/gioi-dau-tu-ky-vong-gi-vao-thuong-dinh-my-trung-5073144.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Tiền lớn chọn lọc, chuyên gia chỉ tên nhóm cổ phiếu xếp hạng cao trên thị trường</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Trong bối cảnh dòng tiền tiếp tục ưu tiên các cổ phiếu có sức mạnh vượt trội, chuyên gia ABS đã tiến hành lọc ra các nhóm ngành và cổ phiếu có mức độ mạnh nhất so với thị trường chung.</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 00:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/tien-lon-chon-loc-chuyen-gia-chi-ten-nhom-co-phieu-xep-hang-cao-tren-thi-truong-188260512213550455.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>VN-Index áp sát đỉnh lịch sử, CTCK cảnh báo kịch bản “xanh vỏ đỏ lòng”</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>VNDirect khuyến nghị chiến lược giao dịch linh hoạt, tận dụng cơ hội chốt lời quanh vùng đỉnh và xem xét giải ngân trở lại nếu chỉ số về vùng hỗ trợ quanh 1.820 điểm.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 00:04:00 +0700</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/vn-index-ap-sat-dinh-lich-su-ctck-canh-bao-kich-ban-xanh-vo-do-long-188260512212732752.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Một công ty chứng khoán vốn nghìn tỷ bị phạt nặng</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Chứng khoán Bảo Minh bị xử phạt tổng cộng 780.000.000 đồng do hàng loạt sai phạm.</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Wed, 13 May 26 00:02:00 +0700</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/mot-cong-ty-chung-khoan-von-nghin-ty-bi-phat-nang-188260512212628665.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Thị trường đang tìm điểm cân bằng mới</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>VnEconomy giới thiệu nhận định v#224; khuyến nghị đầu tư của một số c#244;ng ty chứng kho#225;n về diễn biến thị trường ng#224;y 13/5/2026</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 15:36:11 GMT</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/thi-truong-dang-tim-diem-can-bang-moi.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Quy mô tài sản truyền thống lên tới 1,6 nghìn tỷ USD, Việt Nam có tiềm năng lớn mã hóa tài sản thực</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Chuyên gia tài chính cấp cao đến từ Singapore cho rằng khung pháp lý và sự ủng hộ từ Chính phủ sẽ tiếp tục đóng vai trò quan trọng trong quá trình phát triển của thị trường tài sản mã hóa.</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 26 21:23:00 +0700</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/quy-mo-tai-san-truyen-thong-len-toi-16-nghin-ty-usd-viet-nam-co-tiem-nang-lon-ma-hoa-tai-san-thuc-188260512212342162.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>136 tỷ USD đầu tư cho các dự án điện giai đoạn 2026-2030, cổ phiếu nào hưởng lợi?</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Quyết định số 1509/QĐ-BCT của Bộ C#244;ng Thương đưa ra kế hoạch đầu tư lớn cho giai đoạn 2026- 2030, bao gồm 118 tỷ USD (23,6 tỷ USD/năm) cho sản xuất năng lượng v#224; 18 tỷ USD (3,6 tỷ USD/năm) cho lưới điện.</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 12:02:19 GMT</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/136-ty-usd-dau-tu-cho-cac-du-an-dien-giai-doan-2026-2030-co-phieu-nao-huong-loi.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Vietstock Daily 13/05/2026: Thận trọng trở lại</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>VN-Index hồi phục nhưng khối lượng giao dịch sụt giảm xuống dưới mức trung bình 20 ngày cho thấy tâm lý thận trọng của nhà đầu tư. Chỉ báo Stochastic Oscillator đã cắt xuống đường signal trong vùng overbought nên tình trạng rung lắc nhiều khả năng sẽ còn tiếp diễn trong những phiên tới.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 18:17:00 +0700</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/vietstock-daily-13052026-than-trong-tro-lai-1636-1441621.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Kiểm soát hoạt động của người hành nghề môi giới chứng khoán trên mạng xã hội</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Cần rà soát hoạt động của môi giới chứng khoán nhằm bảo đảm không thực hiện những hoạt động khuyến nghị, tư vấn vượt quá phạm vi.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 26 17:52:00 +0700</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/kiem-soat-hoat-dong-cua-nguoi-hanh-nghe-moi-gioi-chung-khoan-tren-mang-xa-hoi-188260512175208987.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Tự doanh CTCK liên tục bán ra hàng trăm tỷ đồng một cổ phiếu họ Gelex</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Tự doanh CTCK bán ròng 164 tỷ đồng trên HOSE.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 26 17:48:00 +0700</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/tu-doanh-ctck-lien-tuc-ban-ra-hang-tram-ty-dong-mot-co-phieu-ho-gelex-188260512174822907.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Đại diện UBCKNN: Khi nào có sàn giao dịch tài sản mã hoá đầu tiên phụ thuộc hoàn toàn vào năng lực của doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Liên quan tới lộ trình triển khai thị trường tài sản mã hóa chính thức, ông Hòa cho biết tiến độ hiện nay không phụ thuộc vào cơ quan quản lý mà phụ thuộc chủ yếu vào năng lực của doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 26 16:53:00 +0700</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>https://cafef.vn/dai-dien-ubcknn-bao-gio-co-san-giao-dich-tai-san-ma-hoa-dau-tien-phu-thuoc-hoan-toan-vao-nang-luc-cua-doanh-nghiep-188260512165347989.chn</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Nhịp đập Thị trường 12/05: Áp lực bán hạ nhiệt, VN-Index trở lại vùng 1,900</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Thị trường thót tim với pha giảm mạnh của VIC trong ATC, tuy vậy, mọi thứ nhanh chóng qua đi. Kết phiên, VN-Index dừng ở 1,901.1 điểm. HNX-Index có một phiên tích cực khi tăng tới hơn 5 điểm, tương ứng mức 2%.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 16:52:00 +0700</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/nhip-dap-thi-truong-1205-ap-luc-ban-ha-nhiet-vn-index-tro-lai-vung-1900-1636-1441235.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Doanh nghiệp Trung Quốc thâu tóm 'ông lớn' thuốc kháng sinh Imexpharm</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Lian SGP Holding thuộc tập đoàn Livzon Pharmaceutical (Trung Quốc) vừa mua 68% vốn và trở thành cổ đông lớn nhất của doanh nghiệp đứng đầu mảng thuốc kháng sinh Imexpharm.</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 16:21:11 +0700</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/doanh-nghiep-trung-quoc-thau-tom-ong-lon-thuoc-khang-sinh-imexpharm-5073089.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Cổ phiếu tầm trung tăng tốt, VN-Index có “đổi trụ” thành công?</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Những nỗ lực phục hồi về cuối phi#234;n vẫn kh#244;ng đủ để đổi m#224;u gi#225; nh#243;m cổ phiếu vốn h#243;a lớn nhất. Tuy nhi#234;n kh#225; nhiều blue-chips tầm trung cũng như cổ phiếu vừa v#224; nhỏ tăng gi#225; đ#227; b#249; lại phần n#224;o, duy tr#236; sắc xanh cho VN-Index.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 08:25:30 GMT</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/co-phieu-tam-trung-tang-tot-vn-index-co-doi-tru-thanh-cong.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Có thể chính thức khởi động thị trường tài sản mã hóa vào quý 3/2026</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>“Ch#250;ng t#244;i tin rằng sớm nhất trong qu#253; 3 sẽ c#243; những hoạt động ch#237;nh thức đầu ti#234;n của thị trường t#224;i sản m#227; h#243;a tại Việt Nam với c#225;c tổ chức cung cấp dịch vụ dưới cơ chế quản l#253; an to#224;n, minh bạch”...</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 07:09:47 GMT</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/co-the-chinh-thuc-khoi-dong-thi-truong-tai-san-ma-hoa-vao-quy-32026.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Nghiên cứu lập sàn giao dịch chứng khoán cho các startup</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Trong nỗ lực ho#224;n thiện hệ sinh th#225;i đổi mới s#225;ng tạo, Bộ T#224;i ch#237;nh đang nghi#234;n cứu cơ chế thiết lập một thị trường chứng kho#225;n ri#234;ng biệt d#224;nh cho c#225;c doanh nghiệp khởi nghiệp (startup) huy động vốn….</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 06:54:12 GMT</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/nghien-cuu-lap-san-giao-dich-chung-khoan-cho-cac-startup.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Một công ty chứng khoán hạ dự báo tăng trưởng VN-Index do rủi ro bên ngoài</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Dự b#225;o VN-Index đ#243;ng cửa tại 1.967 điểm, tăng 10,2% so với năm 2025 thấp hơn mức dự b#225;o 2.100 điểm được đưa ra đầu năm do phản #225;nh rủi ro bất định từ b#234;n ngo#224;i.</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 06:46:27 GMT</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/mot-cong-ty-chung-khoan-ha-du-bao-tang-truong-vn-index-do-rui-ro-ben-ngoai.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Phân tích kỹ thuật phiên chiều 12/05: Tiếp tục điều chỉnh</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>VN-Index tiếp tục điều chỉnh sau khi không thể vượt qua đỉnh cũ tháng 01/2026 (tương đương vùng 1,900-1,920 điểm). HNX-Index tiếp tục tăng điểm và đang kiểm tra lại đường SMA 50 ngày trong bối cảnh khối lượng giao dịch trồi sụt thất thường.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 13:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/phan-tich-ky-thuat-phien-chieu-1205-tiep-tuc-dieu-chinh-585-1441309.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Vietstock</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UBCKNN yêu cầu CTCK giám sát việc nhân viên "phím hàng" trên mạng xã hội</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>UBCKNN vừa có văn bản gửi các công ty chứng khoán, yêu cầu tăng cường rà soát và giám sát hoạt động của người hành nghề chứng khoán trên mạng xã hội, trong bối cảnh các nội dung phân tích, khuyến nghị đầu tư ngày càng phổ biến trên các nền tảng mạng xã hội.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 12:52:33 +0700</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>http://vietstock.vn/2026/05/ubcknn-yeu-cau-ctck-giam-sat-viec-nhan-vien-phim-hang-tren-mang-xa-hoi-143-1441306.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Thanh khoản hụt hơi, cổ phiếu trụ tiếp tục giảm mạnh</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Mặc d#249; độ rộng chỉ số s#225;ng nay kh#244;ng qu#225; k#233;m nhưng ảnh hưởng từ c#225;c cổ phiếu trụ lại khiến VN-Index tổn thất nặng. Chỉ số giảm th#234;m 0,83% (-15,68 điểm), x#225;c nhận nỗ lực vượt đỉnh thất bại.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 05:08:37 GMT</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/thanh-khoan-hut-hoi-co-phieu-tru-tiep-tuc-giam-manh.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>EU rót hơn 230 tỷ USD vào pin, xe điện để giảm phụ thuộc Trung Quốc</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Châu Âu và Thụy Sĩ đầu tư 235 tỷ USD vào chuỗi cung ứng pin, xe điện và trạm sạc, nhằm định hình hệ sinh thái và giảm phụ thuộc vào Trung Quốc.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 12:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/eu-rot-hon-230-ty-usd-vao-pin-xe-dien-de-giam-phu-thuoc-trung-quoc-5072856.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Thị trường hiện tại là “mỏ vàng” cho nhà đầu tư kiên nhẫn, nhiều cổ phiếu tốt và giá rất thấp</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Lời khuy#234;n cho nh#224; đầu tư đ#243; l#224; đừng qu#225; lo lắng về việc gi#225; chưa tăng ngay. Trong đầu tư, gi#225; cả sớm muộn cũng sẽ đồng quy với gi#225; trị nội tại. Việc mua được “h#224;ng tốt” ở “mức gi#225; thấp” l#224; lợi thế lớn nhất để c#243; bi#234;n lợi nhuận vượt trội trong tương lai.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 03:21:22 GMT</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/thi-truong-hien-tai-la-mo-vang-cho-nha-dau-tu-kien-nhan-nhieu-co-phieu-tot-va-gia-rat-thap.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Các ETF ngoại tiếp tục rút ròng trên thị trường Việt Nam</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>C#225;c quỹ ETF ngoại ghi nhận d#242;ng tiền r#250;t r#242;ng hơn 121 tỷ đồng, tập trung hầu hết ở quỹ Fubon FTSE Vietnam ETF -226,6 tỷ đồng.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 02:52:20 GMT</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/cac-etf-ngoai-tiep-tuc-rut-rong-tren-thi-truong-viet-nam.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Top 3 nhóm ngành mạnh nhất so với thị trường chung</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Trong bối cảnh d#242;ng tiền t#236;m kiếm đến c#225;c cổ phiếu mạnh nhất, ABS lọc ra c#225;c nh#243;m ng#224;nh v#224; cổ phiếu mạnh nhất so với thị trường chung.</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Tue, 12 May 2026 00:00:59 GMT</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/top-3-nhom-nganh-manh-nhat-so-voi-thi-truong-chung.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>VN-Index mất mốc 1900 điểm, nhà đầu tư cẩn trọng trước điều chỉnh</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>VnEconomy giới thiệu nhận định v#224; khuyến nghị đầu tư của một số c#244;ng ty chứng kho#225;n về diễn biến thị trường ng#224;y 12/5/2026</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 15:26:44 GMT</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/vn-index-mat-moc-1900-diem-nha-dau-tu-can-trong-truoc-dieu-chinh.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>'Cá voi' Bitcoin trị giá 40 triệu USD thức giấc</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sau hơn 10 năm nắm giữ, một nhà đầu tư đã chuyển lượng Bitcoin trị giá 40 triệu USD sang ví mới trong bối cảnh tiền số phục hồi.</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 21:19:05 +0700</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/ca-voi-bitcoin-tri-gia-40-trieu-usd-thuc-giac-5072749.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Cá nhân tiếp tục mua ròng mạnh khi VN-Index rớt khỏi mốc 1.900 điểm</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Nh#224; đầu tư c#225; nh#226;n h#244;m nay mua r#242;ng 744,7 tỷ đồng trong đ#243; nh#224; đầu tư trong nước mua r#242;ng khớp lệnh 607 tỷ đồng. T#237;nh ri#234;ng khớp lệnh, nh#224; đầu tư c#225; nh#226;n mua r#242;ng chủ yếu l#224; ng#224;nh Bất động sản.</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 12:46:58 GMT</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>1</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/ca-nhan-tiep-tuc-mua-rong-manh-khi-vn-index-rot-khoi-moc-1900-diem.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>“Trùm” bán khống Michael Burry: Thị trường bây giờ giống những tháng cuối của bong bóng dotcom</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>quot;C#243; cảm gi#225;c b#226;y giờ đang giống như những th#225;ng cuối c#249;ng của bong b#243;ng v#224;o năm 1999-2000quot;, nh#224; b#225;n khống nổi tiếng Michael Burry nhận định...</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 10:58:53 GMT</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>1</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/trum-ban-khong-michael-burry-thi-truong-bay-gio-giong-nhung-thang-cuoi-cua-bong-bong-dotcom.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Blog chứng khoán: Bữa tiệc vắng khách</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>C#225;c cổ phiếu trụ dẫn dắt quay đầu giảm h#244;m nay tạo hiệu ứng ti#234;u cực tr#234;n diện rộng khi nh#224; đầu tư đ#227; chịu đựng qu#225; đủ t#236;nh trạng “xanh vỏ đỏ l#242;ng” những phi#234;n gần đ#226;y.</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 09:28:46 GMT</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>1</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/blog-chung-khoan-bua-tiec-vang-khach.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>VN-Index giảm gần 20 điểm phiên đầu tuần</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Bốn cổ phiếu liên quan đến Vingroup đều giảm, dao động 1-6,5%, trở thành tác nhân chính khiến VN-Index mất gần 20 điểm trong phiên đầu tuần.</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 15:49:54 +0700</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>1</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/vn-index-giam-gan-20-diem-phien-dau-tuan-5072618.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Chỉ số “méo mó”, thị trường cần sự đồng thuận của dòng tiền</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>T#236;nh trạng lệch pha giữa chỉ số v#224; mặt bằng chung n#224;y đang l#224; chủ đề được giới đầu tư theo d#245;i chặt. Nhiều #253; kiến cho rằng, nếu độ rộng v#224; thanh khoản kh#244;ng sớm cải thiện, rủi ro điều chỉnh kỹ thuật quanh v#249;ng đỉnh sẽ tăng l#234;n.</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 07:08:33 GMT</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>1</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/chi-so-meo-mo-thi-truong-can-su-dong-thuan-cua-dong-tien.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>VN-Index vượt mốc 1920 điểm, cổ phiếu chứng khoán khởi sắc trở lại</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Tuy độ rộng thị trường s#225;ng nay vẫn nghi#234;ng hẳn về ph#237;a giảm gi#225; nhưng sức mạnh từ nh#243;m trụ vẫn đủ sức “gồng g#225;nh” VN-Index v#224; đẩy chỉ số l#234;n mức 1921,29 điểm. Như vậy VN-Index đ#227; ho#224;n to#224;n vượt l#234;n tr#234;n v#249;ng đỉnh lịch sử, nhưng thị trường chung kh#244;ng c#243; qu#225;n t#237;nh b#249;ng nổ.</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 05:10:22 GMT</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>1</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/vn-index-vuot-moc-1920-diem-co-phieu-chung-khoan-khoi-sac-tro-lai.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Tổ chức trong nước bán ròng gần 2.000 tỷ tuần qua</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Nh#224; đầu tư tổ chức trong nước b#225;n r#242;ng 1875.3 tỷ đồng, t#237;nh ri#234;ng khớp lệnh th#236; họ b#225;n r#242;ng 0.6 tỷ đồng.</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 03:23:29 GMT</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>1</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/to-chuc-trong-nuoc-ban-rong-gan-2000-ty-tuan-qua.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Cơn sốt hợp đồng tài chính khoai tây ở châu Âu giữa chiến tranh Mỹ - Iran</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Một cơn sốt đầu cơ khoai t#226;y đang diễn ra ở ch#226;u #194;u d#249; hiện tại, khu vực n#224;y đang đối mặt với t#236;nh trạng dư thừa nguồn cung n#244;ng sản n#224;y...</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 02:33:57 GMT</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>1</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/con-sot-hop-dong-tai-chinh-khoai-tay-o-chau-au-giua-chien-tranh-my-iran.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>12,8 nghìn tỷ đồng trái phiếu có vấn đề trong quý 1/2026, chủ yếu ở nhóm Bất động sản</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Tỷ lệ tr#225;i phiếu c#243; vấn đề ph#225;t sinh mới đ#227; giảm từ năm 2024, cho thấy khả năng trả nợ cũng như năng lực t#224;i ch#237;nh của c#225;c tổ chức ph#225;t h#224;nh đ#227; cải thiện đ#225;ng kể trong c#225;c năm gần đ#226;y.</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 02:31:04 GMT</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>1</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/128-nghin-ty-dong-trai-phieu-co-van-de-trong-quy-12026-chu-yeu-o-nhom-bat-dong-san.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>VN-Index được dự đoán sớm vượt 2.000 điểm</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Nhiều nhóm phân tích cho rằng VN-Index tháng này có thể vượt 2.000 điểm nhờ lực kéo từ cổ phiếu trụ và thanh khoản dồi dào.</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Mon, 11 May 2026 00:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>1</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/vn-index-duoc-du-doan-som-vuot-2-000-diem-5072145.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Sổ đỏ cấp sai quy định được xem xét điều chỉnh, nộp bổ sung thuế</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Các dự án được cấp sổ đỏ sai quy định trước đây sẽ được xem xét điều chỉnh và nộp bổ sung nghĩa vụ tài chính, theo cơ chế đặc thù của Chính phủ.</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Sun, 10 May 2026 17:40:04 +0700</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>1</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/so-do-cap-sai-quy-dinh-duoc-xem-xet-dieu-chinh-nop-bo-sung-thue-5072135.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Đề xuất doanh nghiệp nộp thuế thay người gom ve chai, phế liệu</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>VCCI đề nghị Bộ Tài chính bổ sung cơ chế khai, nộp thuế thay với hộ kinh doanh ve chai, đồng nát và sửa cách tính thuế với mô hình tài xế công nghệ.</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Sun, 10 May 2026 12:48:02 +0700</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/de-xuat-doanh-nghiep-nop-thue-thay-nguoi-gom-ve-chai-phe-lieu-5072084.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Xu thế dòng tiền: VN-Index lên đỉnh cao lịch sử mới, thị trường vẫn kém vui</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Thị trường tuần đầu th#225;ng 5 đ#227; x#225;c lập đỉnh cao lịch sử mới của VN-Index khi đ#243;ng cửa tại 1915,37 điểm. Chỉ số cũng ghi nhận tuần tăng thứ 7 li#234;n tiếp. D#249; vậy hiện tượng “xanh vỏ đỏ l#242;ng” gần như trọn tuần khi kiến nh#224; đầu tư kh#244;ng c#243; trải nghiệm t#237;ch cực.</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Sun, 10 May 2026 03:13:57 GMT</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/xu-the-dong-tien-vn-index-len-dinh-cao-lich-su-moi-thi-truong-van-kem-vui.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Rủi ro với mặt bằng chung cổ phiếu giảm đi đáng kể</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Yếu tố quan trọng nhất m#224; thị trường thế giới đang tr#244;ng chờ l#224; triển vọng Mỹ v#224; Iran sớm đạt được thỏa thuận về việc chấm dứt xung đột, rất khả thi...</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Sun, 10 May 2026 03:03:32 GMT</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>1</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/rui-ro-voi-mat-bang-chung-co-phieu-giam-di-dang-ke.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>VN-Index đã vượt đỉnh, nhưng vẫn cần thêm đồng thuận để hoàn toàn bật lên khỏi vùng 1900 – 1920</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>VnEconomy giới thiệu nhận định v#224; khuyến nghị đầu tư của một số c#244;ng ty chứng kho#225;n về diễn biến thị trường tuần từ 11-15/5/2026.</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Sun, 10 May 2026 03:02:08 GMT</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>1</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/vn-index-da-vuot-dinh-nhung-van-can-them-dong-thuan-de-hoan-toan-bat-len-khoi-vung-1900-1920.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Kinh tế Việt - Ấn: Rộng cửa đón tỷ USD</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Chuyến thăm Ấn Độ của Tổng Bí thư, Chủ tịch nước Tô Lâm mở ra dư địa thúc đẩy thương mại song phương, hướng tới mục tiêu 25 tỷ USD vào năm 2030.</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Sun, 10 May 2026 07:00:07 +0700</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/kinh-te-viet-an-rong-cua-don-ty-usd-5072031.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Việt Nam chi gần tỷ USD nhập hạt điều trong một tháng</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Là nước xuất khẩu điều nhân lớn nhất thế giới, nhưng riêng tháng 4, các doanh nghiệp Việt đã chi gần 943 triệu USD để nhập khẩu điều thô.</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 19:58:16 +0700</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/viet-nam-chi-gan-ty-usd-nhap-hat-dieu-trong-mot-thang-5071916.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>VnExpress Business</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Có nên bán nhà Hà Nội khi giá đã giảm 1 tỷ đồng?</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Theo chuyên gia, thị trường bất động sản không trả tiền theo "ký ức" mà theo khả năng, cần đưa ra giá bán phù hợp với thanh khoản thực tế.</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Sat, 09 May 2026 13:00:55 +0700</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>https://vnexpress.net/co-nen-ban-nha-ha-noi-khi-gia-da-giam-1-ty-dong-5071849.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>VNeconomy</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Blog chứng khoán: Cơ hội ngày càng mỏng</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>T#226;m l#253; ch#225;n nản d#226;ng cao hơn trong phi#234;n cuối tuần bất chấp VNI thực sự đ#243;ng cửa ở đỉnh cao lịch sử mới. Độ rộng rất ti#234;u cực v#224; cổ phiếu bị #233;p xuống bi#234;n độ kh#225; rộng trong phi#234;n x#225;c nhận b#234;n b#225;n đ#227; tạo #225;p lực đủ lớn.</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Fri, 08 May 2026 09:36:08 GMT</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>https://vneconomy.vn/blog-chung-khoan-co-hoi-ngay-cang-mong-1291631.htm</t>
         </is>
       </c>
     </row>

</xml_diff>